<commit_message>
Daily pipeline 2026-06-29: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,18 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -548,21 +544,13 @@
           <t>other</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M2" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
@@ -571,76 +559,56 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46186.8905787037</v>
+        <v>46190.37179398148</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M3" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N3" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O3" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -651,53 +619,65 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46160.52664351852</v>
+        <v>46186.8905787037</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K4" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N4" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -708,61 +688,53 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K5" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O5" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -773,57 +745,61 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K6" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="N6" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -834,7 +810,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -845,7 +821,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -857,14 +833,14 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K7" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
@@ -874,17 +850,17 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -895,61 +871,57 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K8" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -960,23 +932,25 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B9" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -987,30 +961,32 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K9" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1021,65 +997,57 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N10" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J10" t="n">
+        <v>603</v>
+      </c>
+      <c r="K10" t="n">
+        <v>603</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1090,12 +1058,10 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>N</t>
@@ -1103,48 +1069,54 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>585</v>
-      </c>
-      <c r="K11" t="n">
-        <v>869</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N11" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1184,10 +1156,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K12" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1202,7 +1174,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R12" t="inlineStr"/>
@@ -1350,11 +1322,11 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" s="1" t="n">
-        <v>46052</v>
+        <v>46050</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1363,7 +1335,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1379,15 +1351,15 @@
         </is>
       </c>
       <c r="J15" t="n">
+        <v>303</v>
+      </c>
+      <c r="K15" t="n">
         <v>585</v>
-      </c>
-      <c r="K15" t="n">
-        <v>869</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" s="1" t="n">
-        <v>46050</v>
+        <v>46045</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
@@ -1397,14 +1369,14 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>11'6" draft, 6 barges wide</t>
+          <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1415,12 +1387,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" s="1" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>N</t>
@@ -1428,48 +1398,54 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>303</v>
-      </c>
-      <c r="K16" t="n">
-        <v>585</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N16" s="1" t="n">
-        <v>46045</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1480,25 +1456,23 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" s="1" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1509,32 +1483,30 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>585</v>
+        <v>538.7</v>
       </c>
       <c r="K17" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1545,10 +1517,12 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" s="1" t="n">
+        <v>46045</v>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>N</t>
@@ -1556,54 +1530,48 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M18" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J18" t="n">
+        <v>303</v>
+      </c>
+      <c r="K18" t="n">
+        <v>869</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O18" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46037</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1614,23 +1582,25 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46033.86975694444</v>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" s="1" t="n">
+        <v>46037</v>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0106-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1641,163 +1611,35 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K19" t="n">
-        <v>538.7</v>
+        <v>869</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" s="1" t="n">
+        <v>46034</v>
+      </c>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46037.50987268519</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" s="1" t="n">
-        <v>46045</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0003-26</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>303</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" s="1" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46033.86975694444</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" s="1" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0106-26</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>303</v>
-      </c>
-      <c r="K21" t="n">
-        <v>869</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" s="1" t="n">
-        <v>46034</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-06-30: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,29 +555,29 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -585,21 +585,13 @@
           <t>other</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M3" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
@@ -608,76 +600,56 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46186.8905787037</v>
+        <v>46190.37179398148</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M4" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N4" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -688,53 +660,65 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46160.52664351852</v>
+        <v>46186.8905787037</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K5" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N5" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -745,61 +729,53 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K6" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O6" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -810,57 +786,61 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K7" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="N7" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -871,7 +851,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
@@ -882,7 +862,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -894,14 +874,14 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K8" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
@@ -911,17 +891,17 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -932,61 +912,57 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K9" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -997,23 +973,25 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B10" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1024,30 +1002,32 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K10" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1058,65 +1038,57 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N11" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O11" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J11" t="n">
+        <v>603</v>
+      </c>
+      <c r="K11" t="n">
+        <v>603</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1127,12 +1099,10 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B12" t="inlineStr"/>
-      <c r="C12" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>N</t>
@@ -1140,48 +1110,54 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>585</v>
-      </c>
-      <c r="K12" t="n">
-        <v>869</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N12" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1192,11 +1168,11 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" s="1" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1205,7 +1181,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1221,7 +1197,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K13" t="n">
         <v>869</v>
@@ -1229,7 +1205,7 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
@@ -1239,14 +1215,14 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1257,11 +1233,11 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1270,7 +1246,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1289,17 +1265,17 @@
         <v>303</v>
       </c>
       <c r="K14" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1311,7 +1287,7 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1322,11 +1298,11 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1335,7 +1311,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1359,7 +1335,7 @@
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" s="1" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
@@ -1376,7 +1352,7 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1387,10 +1363,12 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>N</t>
@@ -1398,54 +1376,48 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J16" t="n">
+        <v>303</v>
+      </c>
+      <c r="K16" t="n">
+        <v>585</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O16" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1456,57 +1428,65 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K17" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N17" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1517,25 +1497,23 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1546,32 +1524,30 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K18" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1582,11 +1558,11 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="1" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1595,7 +1571,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1619,12 +1595,12 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" s="1" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1636,10 +1612,75 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>303</v>
+      </c>
+      <c r="K20" t="n">
+        <v>869</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Set drone-flight safety zone notice to confirmed=N (hide from map)
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -49,9 +48,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -528,12 +528,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>46203.47113425926</v>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0041-26</t>
@@ -544,37 +541,26 @@
           <t>other</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
           <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>46202.62762731482</v>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>CGD-H BNM 0073-26</t>
@@ -585,23 +571,11 @@
           <t>other_NA</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
           <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
@@ -614,11 +588,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>46198.35914351852</v>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>N</t>
@@ -634,19 +606,6 @@
           <t>cancellation</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
           <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
@@ -659,11 +618,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>46190.37179398148</v>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -684,22 +641,12 @@
           <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>28.8597396564073</v>
       </c>
       <c r="M5" t="n">
         <v>-94.1676102718865</v>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
           <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
@@ -712,13 +659,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>46186.8905787037</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
         <v>46199</v>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>N</t>
@@ -734,7 +680,6 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Midway</t>
@@ -745,22 +690,18 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>35.07917</v>
       </c>
       <c r="M6" t="n">
         <v>-90.17319999999999</v>
       </c>
-      <c r="N6" s="1" t="n">
+      <c r="N6" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="O6" s="1" t="n">
+      <c r="O6" s="2" t="n">
         <v>46195</v>
       </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>Mouth of McKellar Lake</t>
@@ -783,11 +724,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>46160.52664351852</v>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Y</t>
@@ -803,8 +742,6 @@
           <t>shoaling</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -816,13 +753,6 @@
       <c r="K7" t="n">
         <v>777.7</v>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr">
         <is>
           <t>Proceed with caution</t>
@@ -840,11 +770,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>46146.4284375</v>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>N</t>
@@ -860,8 +788,6 @@
           <t>other_dredging</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>ARK</t>
@@ -873,16 +799,12 @@
       <c r="K8" t="n">
         <v>155.9</v>
       </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" s="1" t="n">
+      <c r="N8" s="2" t="n">
         <v>46146</v>
       </c>
-      <c r="O8" s="1" t="n">
+      <c r="O8" s="2" t="n">
         <v>46188</v>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
@@ -905,11 +827,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>46119.48518518519</v>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -925,8 +845,6 @@
           <t>shoaling</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -938,12 +856,6 @@
       <c r="K9" t="n">
         <v>686</v>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
           <t>Along RDB</t>
@@ -966,11 +878,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>46093.45828703704</v>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>N</t>
@@ -986,8 +896,6 @@
           <t>other_shoaling</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>ARK</t>
@@ -999,12 +907,6 @@
       <c r="K10" t="n">
         <v>348.7</v>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>Mid channel</t>
@@ -1027,13 +929,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>46065.67140046296</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
         <v>46070</v>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>N</t>
@@ -1049,8 +950,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1062,12 +961,9 @@
       <c r="K11" t="n">
         <v>869</v>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" s="1" t="n">
+      <c r="N11" s="2" t="n">
         <v>46068</v>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1078,8 +974,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
           <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
@@ -1092,11 +986,9 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>46064.87337962963</v>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1112,8 +1004,6 @@
           <t>shoaling</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1125,12 +1015,6 @@
       <c r="K12" t="n">
         <v>603</v>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>400 ft of green buoy line, near RDB</t>
@@ -1153,11 +1037,9 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>46062.51478009259</v>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>N</t>
@@ -1173,7 +1055,6 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Midway</t>
@@ -1184,22 +1065,18 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>35.085769</v>
       </c>
       <c r="M13" t="n">
         <v>-90.10947400000001</v>
       </c>
-      <c r="N13" s="1" t="n">
+      <c r="N13" s="2" t="n">
         <v>46062</v>
       </c>
-      <c r="O13" s="1" t="n">
+      <c r="O13" s="2" t="n">
         <v>46065</v>
       </c>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>Amrize Dock on Mckellar Lake</t>
@@ -1222,11 +1099,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>46058.58436342593</v>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>46068</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -1244,8 +1120,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1257,12 +1131,9 @@
       <c r="K14" t="n">
         <v>869</v>
       </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" s="1" t="n">
+      <c r="N14" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1273,8 +1144,6 @@
           <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
           <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
@@ -1287,11 +1156,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>46051.75101851852</v>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>46061</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -1309,8 +1177,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1322,12 +1188,9 @@
       <c r="K15" t="n">
         <v>869</v>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" s="1" t="n">
+      <c r="N15" s="2" t="n">
         <v>46052</v>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1338,8 +1201,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
           <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
@@ -1352,11 +1213,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>46050.44465277778</v>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -1374,8 +1234,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1387,12 +1245,9 @@
       <c r="K16" t="n">
         <v>585</v>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" s="1" t="n">
+      <c r="N16" s="2" t="n">
         <v>46050</v>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1403,8 +1258,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
@@ -1417,11 +1270,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>46045.53974537037</v>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -1439,8 +1291,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1452,12 +1302,9 @@
       <c r="K17" t="n">
         <v>585</v>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" s="1" t="n">
+      <c r="N17" s="2" t="n">
         <v>46045</v>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1468,8 +1315,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
@@ -1482,11 +1327,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>46042.81428240741</v>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>N</t>
@@ -1502,7 +1345,6 @@
           <t>dredging</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Midway</t>
@@ -1513,22 +1355,18 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>35.0859560963022</v>
       </c>
       <c r="M18" t="n">
         <v>-90.10785143484679</v>
       </c>
-      <c r="N18" s="1" t="n">
+      <c r="N18" s="2" t="n">
         <v>46042.81428240741</v>
       </c>
-      <c r="O18" s="1" t="n">
+      <c r="O18" s="2" t="n">
         <v>46044</v>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>McKellar Lake, near west side of Treasure Island</t>
@@ -1551,11 +1389,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>46037.53365740741</v>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1571,8 +1407,6 @@
           <t>shoaling</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1584,12 +1418,6 @@
       <c r="K19" t="n">
         <v>538.7</v>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>Along LDB</t>
@@ -1612,11 +1440,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>46037.50987268519</v>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>46045</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1634,8 +1461,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1647,12 +1472,9 @@
       <c r="K20" t="n">
         <v>869</v>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" s="1" t="n">
+      <c r="N20" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1663,8 +1485,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
@@ -1677,11 +1497,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>46033.86975694444</v>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>46037</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1699,8 +1518,6 @@
           <t>draft</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1712,12 +1529,9 @@
       <c r="K21" t="n">
         <v>869</v>
       </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" s="1" t="n">
+      <c r="N21" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1728,8 +1542,6 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-05: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -48,10 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,669 +528,782 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="1" t="n">
+        <v>46207.88481481482</v>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0041-26</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
         <v>46203.47113425926</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
         <is>
           <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>46202.62762731482</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>other_NA</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
         <is>
           <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
         <v>46198.35914351852</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>cancellation</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
         <is>
           <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>46190.37179398148</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
         <v>28.8597396564073</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M6" t="n">
         <v>-94.1676102718865</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
         <is>
           <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
         <v>46186.8905787037</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B7" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>dredging</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Midway</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
         <v>35.07917</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M7" t="n">
         <v>-90.17319999999999</v>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="N7" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="O6" s="2" t="n">
+      <c r="O7" s="1" t="n">
         <v>46195</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Mouth of McKellar Lake</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
         <v>46160.52664351852</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>shoaling</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="J8" t="n">
         <v>777.7</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K8" t="n">
         <v>777.7</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
         <is>
           <t>Proceed with caution</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>46146.4284375</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>other_dredging</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
         <is>
           <t>ARK</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="J9" t="n">
         <v>125.4</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K9" t="n">
         <v>155.9</v>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
         <v>46146</v>
       </c>
-      <c r="O8" s="2" t="n">
+      <c r="O9" s="1" t="n">
         <v>46188</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
         <is>
           <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
         <v>46119.48518518519</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>shoaling</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="J10" t="n">
         <v>686</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K10" t="n">
         <v>686</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
         <is>
           <t>Along RDB</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>46093.45828703704</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>other_shoaling</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
         <is>
           <t>ARK</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="J11" t="n">
         <v>348.7</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K11" t="n">
         <v>348.7</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
         <is>
           <t>Mid channel</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
         <v>46065.67140046296</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B12" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="J12" t="n">
         <v>303</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K12" t="n">
         <v>869</v>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
         <is>
           <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
         <v>46064.87337962963</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>shoaling</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="J13" t="n">
         <v>603</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K13" t="n">
         <v>603</v>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
         <is>
           <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Proceed with caution</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
         <v>46062.51478009259</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>dredging</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Midway</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="L13" t="n">
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
         <v>35.085769</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M14" t="n">
         <v>-90.10947400000001</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="N14" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="O13" s="2" t="n">
+      <c r="O14" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
         <is>
           <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
         <v>46058.58436342593</v>
       </c>
-      <c r="C14" s="2" t="n">
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J14" t="n">
+      <c r="J15" t="n">
         <v>585</v>
-      </c>
-      <c r="K14" t="n">
-        <v>869</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0008-26</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>303</v>
       </c>
       <c r="K15" t="n">
         <v>869</v>
       </c>
-      <c r="N15" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" s="1" t="n">
+        <v>46061</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
@@ -1198,12 +1311,14 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1213,11 +1328,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46050.44465277778</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>46052</v>
+      <c r="A16" s="1" t="n">
+        <v>46051.75101851852</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" s="1" t="n">
+        <v>46061</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1226,7 +1342,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1234,6 +1350,8 @@
           <t>draft</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1243,14 +1361,17 @@
         <v>303</v>
       </c>
       <c r="K16" t="n">
-        <v>585</v>
-      </c>
-      <c r="N16" s="2" t="n">
-        <v>46050</v>
-      </c>
+        <v>869</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" s="1" t="n">
+        <v>46052</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1258,9 +1379,11 @@
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1270,11 +1393,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46045.53974537037</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>46050</v>
+      <c r="A17" s="1" t="n">
+        <v>46050.44465277778</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" s="1" t="n">
+        <v>46052</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1283,7 +1407,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1291,6 +1415,8 @@
           <t>draft</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1302,222 +1428,255 @@
       <c r="K17" t="n">
         <v>585</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" s="1" t="n">
+        <v>46050</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" s="1" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>303</v>
+      </c>
+      <c r="K18" t="n">
+        <v>585</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
         <is>
           <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
         <is>
           <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
         <v>46042.81428240741</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>dredging</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
         <is>
           <t>Midway</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="L18" t="n">
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
         <v>35.0859560963022</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M19" t="n">
         <v>-90.10785143484679</v>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="N19" s="1" t="n">
         <v>46042.81428240741</v>
       </c>
-      <c r="O18" s="2" t="n">
+      <c r="O19" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
         <is>
           <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="S19" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>46037.53365740741</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>shoaling</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="n">
+      <c r="J20" t="n">
         <v>538.7</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K20" t="n">
         <v>538.7</v>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
         <is>
           <t>Along LDB</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S20" t="inlineStr">
         <is>
           <t>Transit the area with caution</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
         <v>46037.50987268519</v>
       </c>
-      <c r="C20" s="2" t="n">
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>303</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
-      <c r="N20" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>46033.86975694444</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0106-26</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
@@ -1529,25 +1688,95 @@
       <c r="K21" t="n">
         <v>869</v>
       </c>
-      <c r="N21" s="2" t="n">
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>303</v>
+      </c>
+      <c r="K22" t="n">
+        <v>869</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-06: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -559,14 +559,14 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
@@ -592,38 +592,30 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -639,40 +631,36 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -686,11 +674,15 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -701,40 +693,32 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
@@ -743,7 +727,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -754,67 +738,49 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M7" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N7" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O7" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -825,53 +791,67 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B8" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K8" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -882,61 +862,53 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K9" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -947,57 +919,61 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K10" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1008,37 +984,37 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K11" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -1048,17 +1024,17 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1069,11 +1045,9 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
@@ -1082,48 +1056,46 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K12" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1134,23 +1106,25 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B13" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1161,30 +1135,32 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K13" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="N13" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1195,65 +1171,57 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N14" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O14" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J14" t="n">
+        <v>603</v>
+      </c>
+      <c r="K14" t="n">
+        <v>603</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1264,12 +1232,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>N</t>
@@ -1277,48 +1243,54 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>585</v>
-      </c>
-      <c r="K15" t="n">
-        <v>869</v>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N15" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1329,11 +1301,11 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" s="1" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1342,7 +1314,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1358,7 +1330,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K16" t="n">
         <v>869</v>
@@ -1366,7 +1338,7 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
@@ -1376,14 +1348,14 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1394,11 +1366,11 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1407,7 +1379,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1426,17 +1398,17 @@
         <v>303</v>
       </c>
       <c r="K17" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1448,7 +1420,7 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1459,11 +1431,11 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1472,7 +1444,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1496,7 +1468,7 @@
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" s="1" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
@@ -1513,7 +1485,7 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1524,10 +1496,12 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>N</t>
@@ -1535,54 +1509,48 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J19" t="n">
+        <v>303</v>
+      </c>
+      <c r="K19" t="n">
+        <v>585</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O19" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1593,57 +1561,65 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K20" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O20" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1654,25 +1630,23 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1683,32 +1657,30 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K21" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1719,11 +1691,11 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="1" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1732,7 +1704,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1756,12 +1728,12 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="1" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1773,10 +1745,75 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>303</v>
+      </c>
+      <c r="K23" t="n">
+        <v>869</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-07: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,25 +555,29 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -596,14 +600,14 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
@@ -629,38 +633,30 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -676,40 +672,36 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -723,11 +715,15 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -738,40 +734,32 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -780,7 +768,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -791,67 +779,49 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M8" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N8" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -862,53 +832,67 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B9" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K9" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N9" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -919,61 +903,53 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K10" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -984,57 +960,61 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K11" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="N11" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1045,37 +1025,37 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K12" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1085,17 +1065,17 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1106,11 +1086,9 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
@@ -1119,48 +1097,46 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K13" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1171,23 +1147,25 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1198,30 +1176,32 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K14" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1232,65 +1212,57 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M15" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O15" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J15" t="n">
+        <v>603</v>
+      </c>
+      <c r="K15" t="n">
+        <v>603</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1301,12 +1273,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>N</t>
@@ -1314,48 +1284,54 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>585</v>
-      </c>
-      <c r="K16" t="n">
-        <v>869</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N16" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1366,11 +1342,11 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" s="1" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1379,7 +1355,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1395,7 +1371,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K17" t="n">
         <v>869</v>
@@ -1403,7 +1379,7 @@
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
@@ -1413,14 +1389,14 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1431,11 +1407,11 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1444,7 +1420,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1463,17 +1439,17 @@
         <v>303</v>
       </c>
       <c r="K18" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1485,7 +1461,7 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1496,11 +1472,11 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1509,7 +1485,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1533,7 +1509,7 @@
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" s="1" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
@@ -1550,7 +1526,7 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1561,10 +1537,12 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>N</t>
@@ -1572,54 +1550,48 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M20" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J20" t="n">
+        <v>303</v>
+      </c>
+      <c r="K20" t="n">
+        <v>585</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O20" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1630,57 +1602,65 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K21" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1691,25 +1671,23 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1720,32 +1698,30 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K22" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1756,11 +1732,11 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="1" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1769,7 +1745,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1793,12 +1769,12 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="1" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -1810,10 +1786,75 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>303</v>
+      </c>
+      <c r="K24" t="n">
+        <v>869</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-08: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -557,27 +557,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -596,25 +596,29 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -637,14 +641,14 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
@@ -670,38 +674,30 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -717,40 +713,36 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -764,11 +756,15 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -779,40 +775,32 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M8" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
@@ -821,7 +809,7 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -832,67 +820,49 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M9" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N9" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -903,53 +873,67 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B10" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K10" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N10" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -960,61 +944,53 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K11" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O11" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1025,57 +1001,61 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K12" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="N12" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1086,37 +1066,37 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K13" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1126,17 +1106,17 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1147,11 +1127,9 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
@@ -1160,48 +1138,46 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K14" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1212,23 +1188,25 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B15" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1239,30 +1217,32 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K15" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1273,65 +1253,57 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O16" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J16" t="n">
+        <v>603</v>
+      </c>
+      <c r="K16" t="n">
+        <v>603</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1342,12 +1314,10 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>N</t>
@@ -1355,48 +1325,54 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>585</v>
-      </c>
-      <c r="K17" t="n">
-        <v>869</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N17" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1407,11 +1383,11 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" s="1" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1420,7 +1396,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1436,7 +1412,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K18" t="n">
         <v>869</v>
@@ -1444,7 +1420,7 @@
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
@@ -1454,14 +1430,14 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1472,11 +1448,11 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1485,7 +1461,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1504,17 +1480,17 @@
         <v>303</v>
       </c>
       <c r="K19" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1526,7 +1502,7 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1537,11 +1513,11 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1550,7 +1526,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1574,7 +1550,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" s="1" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
@@ -1591,7 +1567,7 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1602,10 +1578,12 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1613,54 +1591,48 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M21" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J21" t="n">
+        <v>303</v>
+      </c>
+      <c r="K21" t="n">
+        <v>585</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O21" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1671,57 +1643,65 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K22" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M22" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N22" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O22" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1732,25 +1712,23 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1761,32 +1739,30 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K23" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1797,11 +1773,11 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="1" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1810,7 +1786,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1834,12 +1810,12 @@
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" s="1" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -1851,10 +1827,75 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>303</v>
+      </c>
+      <c r="K25" t="n">
+        <v>869</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-11: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46210.47041666666</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -546,9 +546,17 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>110</v>
+      </c>
+      <c r="K2" t="n">
+        <v>118</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -557,27 +565,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46209.69443287037</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -587,9 +595,17 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>110</v>
+      </c>
+      <c r="K3" t="n">
+        <v>117</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -598,27 +614,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46208.56896990741</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -637,25 +653,29 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -674,25 +694,29 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -711,38 +735,30 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -756,42 +772,30 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -805,64 +809,60 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>other_NA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M9" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -873,11 +873,9 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46198.35914351852</v>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
@@ -891,49 +889,25 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>cancellation</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N10" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -944,7 +918,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46160.52664351852</v>
+        <v>46190.37179398148</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
@@ -955,42 +929,38 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>shoaling</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K11" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>28.8597396564073</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-94.1676102718865</v>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1001,9 +971,11 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B12" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
@@ -1012,50 +984,54 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K12" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N12" s="1" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O12" s="1" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1066,7 +1042,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -1077,7 +1053,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1093,10 +1069,10 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K13" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1104,19 +1080,15 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1127,7 +1099,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
@@ -1138,12 +1110,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1154,30 +1126,34 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K14" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="N14" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O14" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1188,25 +1164,23 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1217,32 +1191,30 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K15" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1253,37 +1225,37 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K16" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1293,17 +1265,17 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1314,9 +1286,11 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B17" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
@@ -1325,54 +1299,48 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M17" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J17" t="n">
+        <v>303</v>
+      </c>
+      <c r="K17" t="n">
+        <v>869</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O17" s="1" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1383,25 +1351,23 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1412,32 +1378,30 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K18" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="1" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1448,12 +1412,10 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" s="1" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>N</t>
@@ -1461,48 +1423,54 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>303</v>
-      </c>
-      <c r="K19" t="n">
-        <v>869</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N19" s="1" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1513,11 +1481,11 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="1" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1526,7 +1494,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1542,32 +1510,32 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K20" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" s="1" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1578,11 +1546,11 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" s="1" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1591,7 +1559,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1610,17 +1578,17 @@
         <v>303</v>
       </c>
       <c r="K21" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" s="1" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -1632,7 +1600,7 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1643,10 +1611,12 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" s="1" t="n">
+        <v>46052</v>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>N</t>
@@ -1654,54 +1624,48 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M22" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J22" t="n">
+        <v>303</v>
+      </c>
+      <c r="K22" t="n">
+        <v>585</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O22" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1712,23 +1676,25 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1739,30 +1705,32 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K23" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" s="1" t="n">
+        <v>46045</v>
+      </c>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1773,12 +1741,10 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>N</t>
@@ -1786,48 +1752,54 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>303</v>
-      </c>
-      <c r="K24" t="n">
-        <v>869</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N24" s="1" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O24" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1838,25 +1810,23 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1867,35 +1837,163 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K25" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="1" t="n">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" s="1" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>869</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>303</v>
+      </c>
+      <c r="K27" t="n">
+        <v>869</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr">
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-14: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -552,10 +552,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>110</v>
+        <v>857</v>
       </c>
       <c r="K2" t="n">
-        <v>118</v>
+        <v>867</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
@@ -565,27 +565,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46212.59893518518</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -597,14 +597,14 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K3" t="n">
-        <v>117</v>
+        <v>10.3</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
@@ -614,27 +614,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46210.47041666666</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -644,9 +644,17 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>110</v>
+      </c>
+      <c r="K4" t="n">
+        <v>118</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -655,27 +663,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46209.69443287037</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -685,9 +693,17 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>110</v>
+      </c>
+      <c r="K5" t="n">
+        <v>117</v>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -696,27 +712,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46208.56896990741</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -735,25 +751,29 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -772,25 +792,29 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -809,38 +833,30 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -854,42 +870,30 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -903,64 +907,60 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>other_NA</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -971,11 +971,9 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46198.35914351852</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
@@ -989,49 +987,25 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>cancellation</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N12" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O12" s="1" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1042,7 +1016,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46160.52664351852</v>
+        <v>46190.37179398148</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -1053,42 +1027,38 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>shoaling</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K13" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>28.8597396564073</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-94.1676102718865</v>
+      </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1099,9 +1069,11 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
@@ -1110,50 +1082,54 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K14" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N14" s="1" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O14" s="1" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1164,7 +1140,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
@@ -1175,7 +1151,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1191,10 +1167,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K15" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1202,19 +1178,15 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1225,7 +1197,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
@@ -1236,12 +1208,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1252,30 +1224,34 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K16" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="N16" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1286,25 +1262,23 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1315,32 +1289,30 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K17" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1351,37 +1323,37 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K18" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
@@ -1391,17 +1363,17 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1412,9 +1384,11 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B19" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
@@ -1423,54 +1397,48 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J19" t="n">
+        <v>303</v>
+      </c>
+      <c r="K19" t="n">
+        <v>869</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O19" s="1" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1481,25 +1449,23 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1510,32 +1476,30 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K20" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" s="1" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1546,12 +1510,10 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" s="1" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1559,48 +1521,54 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>303</v>
-      </c>
-      <c r="K21" t="n">
-        <v>869</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N21" s="1" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1611,11 +1579,11 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="1" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1624,7 +1592,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1640,32 +1608,32 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K22" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="1" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1676,11 +1644,11 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="1" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1689,7 +1657,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1708,17 +1676,17 @@
         <v>303</v>
       </c>
       <c r="K23" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="1" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -1730,7 +1698,7 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1741,10 +1709,12 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" s="1" t="n">
+        <v>46052</v>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>N</t>
@@ -1752,54 +1722,48 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M24" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J24" t="n">
+        <v>303</v>
+      </c>
+      <c r="K24" t="n">
+        <v>585</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O24" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1810,23 +1774,25 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1837,30 +1803,32 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K25" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" s="1" t="n">
+        <v>46045</v>
+      </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1871,12 +1839,10 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>N</t>
@@ -1884,48 +1850,54 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>303</v>
-      </c>
-      <c r="K26" t="n">
-        <v>869</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N26" s="1" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O26" s="1" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1936,25 +1908,23 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1965,35 +1935,163 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K27" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="1" t="n">
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" s="1" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>303</v>
+      </c>
+      <c r="K28" t="n">
+        <v>869</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>303</v>
+      </c>
+      <c r="K29" t="n">
+        <v>869</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr">
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-15: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,14 +529,14 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46216.73908564815</v>
+        <v>46217.56884259259</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -546,17 +546,9 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>857</v>
-      </c>
-      <c r="K2" t="n">
-        <v>867</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -565,27 +557,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -597,14 +589,14 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K3" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
@@ -614,27 +606,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -646,14 +638,14 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K4" t="n">
-        <v>118</v>
+        <v>10.3</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
@@ -663,27 +655,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46212.59893518518</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -702,7 +694,7 @@
         <v>110</v>
       </c>
       <c r="K5" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
@@ -712,27 +704,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46210.47041666666</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -742,9 +734,17 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>110</v>
+      </c>
+      <c r="K6" t="n">
+        <v>117</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -753,27 +753,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -794,27 +794,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -833,25 +833,29 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -874,14 +878,14 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -907,38 +911,30 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -954,40 +950,36 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1001,11 +993,15 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1016,40 +1012,32 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
@@ -1058,7 +1046,7 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1069,67 +1057,49 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M14" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N14" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O14" s="1" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1140,53 +1110,67 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B15" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46199</v>
+      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K15" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M15" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N15" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>46195</v>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1197,61 +1181,53 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K16" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O16" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1262,57 +1238,61 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K17" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="N17" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>46188</v>
+      </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1323,37 +1303,37 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K18" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
@@ -1363,17 +1343,17 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1384,11 +1364,9 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
@@ -1397,48 +1375,46 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K19" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1449,23 +1425,25 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>46070</v>
+      </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1476,30 +1454,32 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K20" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" s="1" t="n">
+        <v>46068</v>
+      </c>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1510,65 +1490,57 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M21" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N21" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O21" s="1" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J21" t="n">
+        <v>603</v>
+      </c>
+      <c r="K21" t="n">
+        <v>603</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1579,12 +1551,10 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>N</t>
@@ -1592,48 +1562,54 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>585</v>
-      </c>
-      <c r="K22" t="n">
-        <v>869</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M22" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N22" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O22" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1644,11 +1620,11 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="1" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1657,7 +1633,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1673,7 +1649,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K23" t="n">
         <v>869</v>
@@ -1681,7 +1657,7 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
@@ -1691,14 +1667,14 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1709,11 +1685,11 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="1" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1722,7 +1698,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1741,17 +1717,17 @@
         <v>303</v>
       </c>
       <c r="K24" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -1763,7 +1739,7 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1774,11 +1750,11 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" s="1" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1787,7 +1763,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1811,7 +1787,7 @@
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" s="1" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
@@ -1828,7 +1804,7 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1839,10 +1815,12 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" s="1" t="n">
+        <v>46050</v>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>N</t>
@@ -1850,54 +1828,48 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M26" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J26" t="n">
+        <v>303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>585</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O26" s="1" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1908,57 +1880,65 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K27" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N27" s="1" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O27" s="1" t="n">
+        <v>46044</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1969,25 +1949,23 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1998,32 +1976,30 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K28" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" s="1" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2034,11 +2010,11 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" s="1" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2047,7 +2023,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2071,12 +2047,12 @@
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
       <c r="N29" s="1" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2088,10 +2064,75 @@
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>303</v>
+      </c>
+      <c r="K30" t="n">
+        <v>869</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-27: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -417,126 +429,126 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U30"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date_published</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cancelled_date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>replaced_date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>active?</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>message_id</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>other_notes</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>dredge</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>river</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>mm_low</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>mm_high</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>lon</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>date_start</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>date_end</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>northbound</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>southbound</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>location_details</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>instructions</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>full_memo</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>confirmed</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46217.56884259259</v>
+      <c r="A2" s="2" t="n">
+        <v>46230.45863425926</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0076-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,29 +567,25 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46216.73908564815</v>
+      <c r="A3" s="2" t="n">
+        <v>46230.45790509259</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0082-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -587,17 +595,9 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>857</v>
-      </c>
-      <c r="K3" t="n">
-        <v>867</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -606,27 +606,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46216.4634375</v>
+      <c r="A4" s="2" t="n">
+        <v>46226.71640046296</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -636,17 +636,9 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K4" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -655,27 +647,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LA, TX- GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46213.22780092592</v>
+      <c r="A5" s="2" t="n">
+        <v>46223.66856481481</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -685,17 +677,9 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>110</v>
-      </c>
-      <c r="K5" t="n">
-        <v>118</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -704,47 +688,39 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46212.59893518518</v>
+      <c r="A6" s="2" t="n">
+        <v>46223.49913194445</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>CGD-H BNM 0079-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>110</v>
-      </c>
-      <c r="K6" t="n">
-        <v>117</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -753,27 +729,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46210.47041666666</v>
+      <c r="A7" s="2" t="n">
+        <v>46220.60020833334</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>CGD-H BNM 0078-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -794,27 +770,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46209.69443287037</v>
+      <c r="A8" s="2" t="n">
+        <v>46220.59974537037</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0077-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -835,27 +811,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46208.56896990741</v>
+      <c r="A9" s="2" t="n">
+        <v>46220.59907407407</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -878,21 +854,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46207.88481481482</v>
+      <c r="A10" s="2" t="n">
+        <v>46217.56884259259</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -911,25 +887,29 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>46203.47113425926</v>
+      <c r="A11" s="2" t="n">
+        <v>46216.73908564815</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -939,9 +919,17 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>857</v>
+      </c>
+      <c r="K11" t="n">
+        <v>867</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -956,37 +944,41 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>46202.62762731482</v>
+      <c r="A12" s="2" t="n">
+        <v>46216.4634375</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>10.3</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -995,80 +987,76 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46198.35914351852</v>
+      <c r="A13" s="2" t="n">
+        <v>46213.22780092592</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>110</v>
+      </c>
+      <c r="K13" t="n">
+        <v>118</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>OUACHITA RIVER</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>46190.37179398148</v>
+      <c r="A14" s="2" t="n">
+        <v>46212.59893518518</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1076,326 +1064,216 @@
           <t>other</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>110</v>
+      </c>
+      <c r="K14" t="n">
+        <v>117</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>46199</v>
-      </c>
+      <c r="A15" s="2" t="n">
+        <v>46210.47041666666</v>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M15" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N15" s="1" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O15" s="1" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LA - GULF OF AMERICA</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>46160.52664351852</v>
+      <c r="A16" s="2" t="n">
+        <v>46209.69443287037</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K16" t="n">
-        <v>777.7</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>46146.4284375</v>
+      <c r="A17" s="2" t="n">
+        <v>46208.56896990741</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K17" t="n">
-        <v>155.9</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="1" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O17" s="1" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>46119.48518518519</v>
+      <c r="A18" s="2" t="n">
+        <v>46207.88481481482</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>686</v>
-      </c>
-      <c r="K18" t="n">
-        <v>686</v>
-      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>46093.45828703704</v>
+      <c r="A19" s="2" t="n">
+        <v>46203.47113425926</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>348.7</v>
-      </c>
-      <c r="K19" t="n">
-        <v>348.7</v>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
@@ -1404,82 +1282,58 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>"Possible shoaling," transit area with caution</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>46070</v>
-      </c>
+      <c r="A20" s="2" t="n">
+        <v>46202.62762731482</v>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>303</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" s="1" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1489,58 +1343,42 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>46064.87337962963</v>
+      <c r="A21" s="2" t="n">
+        <v>46198.35914351852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>cancellation</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>603</v>
-      </c>
-      <c r="K21" t="n">
-        <v>603</v>
-      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1550,160 +1388,148 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>46062.51478009259</v>
+      <c r="A22" s="2" t="n">
+        <v>46190.37179398148</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
-        <v>35.085769</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M22" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N22" s="1" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O22" s="1" t="n">
-        <v>46065</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0039-26</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
         <is>
           <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>46058.58436342593</v>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" s="1" t="n">
-        <v>46068</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>SEC LMR BNM 0009-26</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>draft</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>585</v>
-      </c>
-      <c r="K23" t="n">
-        <v>869</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46160.52664351852</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>46051.75101851852</v>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" s="1" t="n">
-        <v>46061</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1714,32 +1540,26 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>303</v>
+        <v>777.7</v>
       </c>
       <c r="K24" t="n">
-        <v>869</v>
+        <v>777.7</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" s="1" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1749,13 +1569,11 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>46050.44465277778</v>
+      <c r="A25" s="2" t="n">
+        <v>46146.4284375</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" s="1" t="n">
-        <v>46052</v>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>N</t>
@@ -1763,48 +1581,50 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>303</v>
+        <v>125.4</v>
       </c>
       <c r="K25" t="n">
-        <v>585</v>
+        <v>155.9</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="1" t="n">
-        <v>46050</v>
-      </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1814,26 +1634,24 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>46045.53974537037</v>
+      <c r="A26" s="2" t="n">
+        <v>46119.48518518519</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" s="1" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1844,32 +1662,30 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K26" t="n">
-        <v>585</v>
+        <v>686</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1879,8 +1695,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>46042.81428240741</v>
+      <c r="A27" s="2" t="n">
+        <v>46093.45828703704</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
@@ -1891,54 +1707,46 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M27" t="n">
-        <v>-90.10785143484679</v>
-      </c>
-      <c r="N27" s="1" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O27" s="1" t="n">
-        <v>46044</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="K27" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1948,24 +1756,26 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>46037.53365740741</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="A28" s="2" t="n">
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1976,30 +1786,32 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K28" t="n">
-        <v>538.7</v>
+        <v>869</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2009,26 +1821,24 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>46037.50987268519</v>
+      <c r="A29" s="2" t="n">
+        <v>46064.87337962963</v>
       </c>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" s="1" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -2039,100 +1849,622 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K29" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" s="1" t="n">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46062.51478009259</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0011-26</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M30" t="n">
+        <v>-90.10947400000001</v>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46058.58436342593</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="2" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0009-26</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>585</v>
+      </c>
+      <c r="K31" t="n">
+        <v>869</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>46061</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46051.75101851852</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" s="2" t="n">
+        <v>46061</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0008-26</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>303</v>
+      </c>
+      <c r="K32" t="n">
+        <v>869</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46050.44465277778</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0007-26</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>303</v>
+      </c>
+      <c r="K33" t="n">
+        <v>585</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>303</v>
+      </c>
+      <c r="K34" t="n">
+        <v>585</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K36" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>303</v>
+      </c>
+      <c r="K37" t="n">
+        <v>869</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
         <is>
           <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr">
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
         <is>
           <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
+    <row r="38">
+      <c r="A38" s="2" t="n">
         <v>46033.86975694444</v>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" s="1" t="n">
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0106-26</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="J38" t="n">
         <v>303</v>
       </c>
-      <c r="K30" t="n">
+      <c r="K38" t="n">
         <v>869</v>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" s="1" t="n">
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr">
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="U38" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-07-30: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46230.45863425926</v>
+        <v>46232.48969907407</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -571,21 +571,21 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46230.45790509259</v>
+        <v>46230.45863425926</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0082-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -604,29 +604,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46226.71640046296</v>
+        <v>46230.45790509259</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>CGD-H BNM 0082-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -647,27 +643,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LA, TX- GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
+          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46223.66856481481</v>
+        <v>46226.71640046296</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -688,32 +684,32 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>LA, TX- GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
+          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46223.49913194445</v>
+        <v>46223.66856481481</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0079-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -729,32 +725,32 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46220.60020833334</v>
+        <v>46223.49913194445</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0078-26</t>
+          <t>CGD-H BNM 0079-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -770,27 +766,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
+          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46220.59974537037</v>
+        <v>46220.60020833334</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0077-26</t>
+          <t>CGD-H BNM 0078-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -811,27 +807,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
+          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46220.59907407407</v>
+        <v>46220.59974537037</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0076-26</t>
+          <t>CGD-H BNM 0077-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -850,18 +846,22 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46217.56884259259</v>
+        <v>46220.59907407407</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
@@ -887,29 +887,25 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46217.56884259259</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -919,17 +915,9 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>857</v>
-      </c>
-      <c r="K11" t="n">
-        <v>867</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -938,27 +926,27 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -970,14 +958,14 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K12" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -987,27 +975,27 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1019,14 +1007,14 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K13" t="n">
-        <v>118</v>
+        <v>10.3</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1036,27 +1024,27 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46212.59893518518</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1075,7 +1063,7 @@
         <v>110</v>
       </c>
       <c r="K14" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
@@ -1085,27 +1073,27 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46210.47041666666</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1115,9 +1103,17 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>110</v>
+      </c>
+      <c r="K15" t="n">
+        <v>117</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1126,27 +1122,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1167,27 +1163,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1206,25 +1202,29 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1247,14 +1247,14 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1280,38 +1280,30 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1327,40 +1319,36 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1374,11 +1362,15 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1389,40 +1381,32 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M22" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
@@ -1431,7 +1415,7 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1442,67 +1426,49 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M23" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N23" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1513,53 +1479,67 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B24" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K24" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1570,61 +1550,53 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K25" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1635,57 +1607,61 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K26" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="N26" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1696,37 +1672,37 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K27" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
@@ -1736,17 +1712,17 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1757,11 +1733,9 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
@@ -1770,48 +1744,46 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K28" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1822,23 +1794,25 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B29" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -1849,30 +1823,32 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K29" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1883,65 +1859,57 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M30" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N30" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J30" t="n">
+        <v>603</v>
+      </c>
+      <c r="K30" t="n">
+        <v>603</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1952,12 +1920,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>N</t>
@@ -1965,48 +1931,54 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>585</v>
-      </c>
-      <c r="K31" t="n">
-        <v>869</v>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M31" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N31" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -2017,11 +1989,11 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2030,7 +2002,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2046,7 +2018,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K32" t="n">
         <v>869</v>
@@ -2054,7 +2026,7 @@
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
@@ -2064,14 +2036,14 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2082,11 +2054,11 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2095,7 +2067,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2114,17 +2086,17 @@
         <v>303</v>
       </c>
       <c r="K33" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -2136,7 +2108,7 @@
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2147,11 +2119,11 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2160,7 +2132,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2184,7 +2156,7 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
@@ -2201,7 +2173,7 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2212,10 +2184,12 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>N</t>
@@ -2223,54 +2197,48 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M35" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J35" t="n">
+        <v>303</v>
+      </c>
+      <c r="K35" t="n">
+        <v>585</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2281,57 +2249,65 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K36" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M36" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O36" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2342,25 +2318,23 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B37" t="inlineStr"/>
-      <c r="C37" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -2371,32 +2345,30 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K37" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2407,11 +2379,11 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2420,7 +2392,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2444,12 +2416,12 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -2461,10 +2433,75 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>303</v>
+      </c>
+      <c r="K39" t="n">
+        <v>869</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-01: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,51 +541,63 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46232.48969907407</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>849</v>
+      </c>
+      <c r="K2" t="n">
+        <v>849</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46230.45863425926</v>
+        <v>46232.48969907407</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -608,21 +620,21 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46230.45790509259</v>
+        <v>46230.45863425926</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0082-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -641,29 +653,25 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46226.71640046296</v>
+        <v>46230.45790509259</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>CGD-H BNM 0082-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -684,27 +692,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>LA, TX- GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
+          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46223.66856481481</v>
+        <v>46226.71640046296</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -725,32 +733,32 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>LA, TX- GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
+          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46223.49913194445</v>
+        <v>46223.66856481481</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0079-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -766,32 +774,32 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46220.60020833334</v>
+        <v>46223.49913194445</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0078-26</t>
+          <t>CGD-H BNM 0079-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -807,27 +815,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
+          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46220.59974537037</v>
+        <v>46220.60020833334</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0077-26</t>
+          <t>CGD-H BNM 0078-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -848,27 +856,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
+          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46220.59907407407</v>
+        <v>46220.59974537037</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0076-26</t>
+          <t>CGD-H BNM 0077-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -887,18 +895,22 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46217.56884259259</v>
+        <v>46220.59907407407</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
@@ -924,29 +936,25 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46217.56884259259</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -956,17 +964,9 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>857</v>
-      </c>
-      <c r="K12" t="n">
-        <v>867</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -975,27 +975,27 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1007,14 +1007,14 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K13" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
@@ -1024,27 +1024,27 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1056,14 +1056,14 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K14" t="n">
-        <v>118</v>
+        <v>10.3</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
@@ -1073,27 +1073,27 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46212.59893518518</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1112,7 +1112,7 @@
         <v>110</v>
       </c>
       <c r="K15" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1122,27 +1122,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46210.47041666666</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1152,9 +1152,17 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>110</v>
+      </c>
+      <c r="K16" t="n">
+        <v>117</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1163,27 +1171,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1204,27 +1212,27 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1243,25 +1251,29 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1284,14 +1296,14 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
@@ -1317,38 +1329,30 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1364,40 +1368,36 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1411,11 +1411,15 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1426,40 +1430,32 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M23" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
@@ -1468,7 +1464,7 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1479,67 +1475,49 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M24" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N24" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1550,53 +1528,67 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K25" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1607,61 +1599,53 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K26" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1672,57 +1656,61 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K27" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1733,37 +1721,37 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K28" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
@@ -1773,17 +1761,17 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1794,11 +1782,9 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
@@ -1807,48 +1793,46 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K29" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1859,23 +1843,25 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B30" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1886,30 +1872,32 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K30" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1920,65 +1908,57 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M31" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N31" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O31" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J31" t="n">
+        <v>603</v>
+      </c>
+      <c r="K31" t="n">
+        <v>603</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1989,12 +1969,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B32" t="inlineStr"/>
-      <c r="C32" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>N</t>
@@ -2002,48 +1980,54 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>585</v>
-      </c>
-      <c r="K32" t="n">
-        <v>869</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M32" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N32" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2054,11 +2038,11 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2067,7 +2051,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2083,7 +2067,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K33" t="n">
         <v>869</v>
@@ -2091,7 +2075,7 @@
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
       <c r="N33" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
@@ -2101,14 +2085,14 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2119,11 +2103,11 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2132,7 +2116,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2151,17 +2135,17 @@
         <v>303</v>
       </c>
       <c r="K34" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -2173,7 +2157,7 @@
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2184,11 +2168,11 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2197,7 +2181,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2221,7 +2205,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
@@ -2238,7 +2222,7 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2249,10 +2233,12 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>N</t>
@@ -2260,54 +2246,48 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M36" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J36" t="n">
+        <v>303</v>
+      </c>
+      <c r="K36" t="n">
+        <v>585</v>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O36" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2318,57 +2298,65 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K37" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2379,25 +2367,23 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2408,32 +2394,30 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K38" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2444,11 +2428,11 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2457,7 +2441,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2481,12 +2465,12 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -2498,10 +2482,75 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>303</v>
+      </c>
+      <c r="K40" t="n">
+        <v>869</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="U40" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-05: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,34 +541,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>849</v>
-      </c>
-      <c r="K2" t="n">
-        <v>849</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -577,64 +569,76 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46232.48969907407</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>849</v>
+      </c>
+      <c r="K3" t="n">
+        <v>849</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46230.45863425926</v>
+        <v>46232.48969907407</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -657,21 +661,21 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46230.45790509259</v>
+        <v>46230.45863425926</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0082-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -690,29 +694,25 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46226.71640046296</v>
+        <v>46230.45790509259</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>CGD-H BNM 0082-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -733,27 +733,27 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LA, TX- GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
+          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46223.66856481481</v>
+        <v>46226.71640046296</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -774,32 +774,32 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>LA, TX- GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
+          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46223.49913194445</v>
+        <v>46223.66856481481</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0079-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -815,32 +815,32 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46220.60020833334</v>
+        <v>46223.49913194445</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0078-26</t>
+          <t>CGD-H BNM 0079-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -856,27 +856,27 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
+          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46220.59974537037</v>
+        <v>46220.60020833334</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0077-26</t>
+          <t>CGD-H BNM 0078-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -897,27 +897,27 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
+          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46220.59907407407</v>
+        <v>46220.59974537037</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0076-26</t>
+          <t>CGD-H BNM 0077-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -936,18 +936,22 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46217.56884259259</v>
+        <v>46220.59907407407</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -973,29 +977,25 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46217.56884259259</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1005,17 +1005,9 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>857</v>
-      </c>
-      <c r="K13" t="n">
-        <v>867</v>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1024,27 +1016,27 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1056,14 +1048,14 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K14" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
@@ -1073,27 +1065,27 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1105,14 +1097,14 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K15" t="n">
-        <v>118</v>
+        <v>10.3</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1122,27 +1114,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46212.59893518518</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1161,7 +1153,7 @@
         <v>110</v>
       </c>
       <c r="K16" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1171,27 +1163,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46210.47041666666</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1201,9 +1193,17 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>110</v>
+      </c>
+      <c r="K17" t="n">
+        <v>117</v>
+      </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1212,27 +1212,27 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1253,27 +1253,27 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1292,25 +1292,29 @@
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1333,14 +1337,14 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
@@ -1366,38 +1370,30 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1413,40 +1409,36 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1460,11 +1452,15 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1475,40 +1471,32 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M24" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
@@ -1517,7 +1505,7 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1528,67 +1516,49 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M25" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N25" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1599,53 +1569,67 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K26" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1656,61 +1640,53 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K27" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1721,57 +1697,61 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K28" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1782,37 +1762,37 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K29" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -1822,17 +1802,17 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1843,11 +1823,9 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
@@ -1856,48 +1834,46 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K30" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1908,23 +1884,25 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -1935,30 +1913,32 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K31" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1969,65 +1949,57 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M32" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N32" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O32" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J32" t="n">
+        <v>603</v>
+      </c>
+      <c r="K32" t="n">
+        <v>603</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2038,12 +2010,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B33" t="inlineStr"/>
-      <c r="C33" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>N</t>
@@ -2051,48 +2021,54 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>585</v>
-      </c>
-      <c r="K33" t="n">
-        <v>869</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N33" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2103,11 +2079,11 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2116,7 +2092,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2132,7 +2108,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K34" t="n">
         <v>869</v>
@@ -2140,7 +2116,7 @@
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
       <c r="N34" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
@@ -2150,14 +2126,14 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2168,11 +2144,11 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2181,7 +2157,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2200,17 +2176,17 @@
         <v>303</v>
       </c>
       <c r="K35" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -2222,7 +2198,7 @@
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2233,11 +2209,11 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2246,7 +2222,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2270,7 +2246,7 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
@@ -2287,7 +2263,7 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2298,10 +2274,12 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>N</t>
@@ -2309,54 +2287,48 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M37" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J37" t="n">
+        <v>303</v>
+      </c>
+      <c r="K37" t="n">
+        <v>585</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2367,57 +2339,65 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K38" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M38" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2428,25 +2408,23 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -2457,32 +2435,30 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K39" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2493,11 +2469,11 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2506,7 +2482,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2530,12 +2506,12 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -2547,10 +2523,75 @@
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>303</v>
+      </c>
+      <c r="K41" t="n">
+        <v>869</v>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-06: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -558,9 +558,17 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,47 +577,39 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>849</v>
-      </c>
-      <c r="K3" t="n">
-        <v>849</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,64 +618,76 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46232.48969907407</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>849</v>
+      </c>
+      <c r="K4" t="n">
+        <v>849</v>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46230.45863425926</v>
+        <v>46232.48969907407</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -698,21 +710,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0081-26 DTG 232000Z JUL 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46230.45790509259</v>
+        <v>46230.45863425926</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0082-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -731,29 +743,25 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0080-26 DTG 201557Z JUL 262. LAUNCH COMPLETE. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46226.71640046296</v>
+        <v>46230.45790509259</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0081-26</t>
+          <t>CGD-H BNM 0082-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -774,27 +782,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LA, TX- GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
+          <t>1. ON 30JUL2026, FROM 0015Z TO 0145Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W,30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISE PERIOD.CANCEL AT//300230Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46223.66856481481</v>
+        <v>46226.71640046296</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0080-26</t>
+          <t>CGD-H BNM 0081-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -815,32 +823,32 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>LA, TX- GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
+          <t>1. DUE TO THE PASSAGE OF TROPICAL STORM BERTHA, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//312000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46223.49913194445</v>
+        <v>46223.66856481481</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0079-26</t>
+          <t>CGD-H BNM 0080-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -856,32 +864,32 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:23/2245Z JUL 26 TO 24/0015Z JUL 2624/2245Z JUL 26 TO 25/0015Z JUL 2625/2245Z JUL 26 TO 26/0015Z JUL 2626/2245Z JUL 26 TO 27/0015Z JUL 2627/2245Z JUL 26 TO 28/0015Z JUL 2628/2245Z JUL 26 TO 29/0015Z JUL 2629/2245Z JUL 26 TO 30/0015Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//300115Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46220.60020833334</v>
+        <v>46223.49913194445</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0078-26</t>
+          <t>CGD-H BNM 0079-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -897,27 +905,27 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA, MS, AL, FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
+          <t>1. AS TROPICAL DEPRESSION TWO APPROACHES, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. STORM SURGE AND WINDS MAY CREATE SHOALS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL WEATHER CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL SUCH TIME THAT WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. BECAUSE OF THE UNCERTAINTY OF STORM MOVEMENTS AND NAVIGATION STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.2. ALL SECTORS SHOULD BROADCAST SPANISH AND VIETNAMESE VERSIONS, AS APPROPRIATE. SECTORS SHOULD UTILIZE THE FOREIGN LANGUAGE INTERPRETER SERVICES.CANCEL AT//240000Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46220.59974537037</v>
+        <v>46220.60020833334</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0077-26</t>
+          <t>CGD-H BNM 0078-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -938,27 +946,27 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
+          <t>THE U.S. NAVY WILL CONDUCT DAILY SURFACE VESSEL TESTS BETWEEN 20JUL2026 AND 26JUL2026, FROM 1000Z TO0100Z, THE FOLLOWING DAY, IN AN AREA BOUND BY APPROXIMATE POSITIONS30-04-34.35N 085-38-54.51W,29-57-37.33N 085-29-18.73W,29-56-19.03N 085-48-57.67W AND29-48-49.06N 085-38-42.90W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//270200Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46220.59907407407</v>
+        <v>46220.59974537037</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0076-26</t>
+          <t>CGD-H BNM 0077-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -977,18 +985,22 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:20/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 2623/2245Z JUL 26 TO 24/0056Z JUL 2624/2245Z JUL 26 TO 25/0056Z JUL 2625/2245Z JUL 26 TO 26/0056Z JUL 2626/2245Z JUL 26 TO 27/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//270156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46217.56884259259</v>
+        <v>46220.59907407407</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -1014,29 +1026,25 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
+          <t>1. CANCEL CGD-H BNM 0076-26 DTG 141212Z JUL 262. UPDATED NOTICE TO FOLLOW. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46217.56884259259</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>CGD-H BNM 0076-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1046,17 +1054,9 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>857</v>
-      </c>
-      <c r="K14" t="n">
-        <v>867</v>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -1065,27 +1065,27 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>TX - GULF OF AMERICA - CARIBBEAN SEA</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. SPACE LAUNCH OPERATIONS, WHICH MAY BE HAZARDOUS TO SURFACE VESSELS, WILL BE CONDUCTED WITHIN PORTIONS OF THE FOLLOWING HAZARD AREAS FOR STARSHIP FLIGHT 13:A. HIGH RISK HAZARD AREA25-11-42N 092-57-51W,25-30-40N 093-52-27W,25-36-20N 094-39-15W,25-41-50N 095-24-24W,26-02-50N 096-34-49W,26-05-00N 096-52-00W,26-04-00N 097-04-00W,26-04-00N 097-10-00W,26-02-00N 097-13-00W,25-58-00N 097-13-00W,25-48-00N 097-05-00W,25-40-49N 096-46-49W,25-00-56N 094-43-27W,24-39-30N 094-07-03W,24-25-19N 093-23-45W,24-29-46N 092-59-49W AND24-51-30N 092-51-26W.B. HAZARD AREA25-58-00N 097-13-00W,26-02-00N 097-13-00W,26-04-00N 097-10-00W,26-04-00N 097-04-00W,26-05-00N 096-52-00W,26-05-00N 096-28-00W,26-01-00N 095-12-00W,25-45-00N 095-04-00W,25-44-00N 094-08-00W,25-35-00N 093-14-00W,25-37-00N 091-58-00W,24-29-00N 090-54-00W,24-06-00N 089-58-00W,22-21-00N 086-21-00W,21-34-00N 085-04-00W,21-04-00N 082-37-00W,20-48-00N 081-43-00W,20-10-00N 080-01-00W,19-19-00N 077-54-00W,19-05-00N 077-36-00W,19-07-00N 078-04-00W,19-29-00N 079-08-00W,19-45-00N 079-44-00W,20-18-00N 081-13-00W,20-34-00N 083-16-00W,21-16-00N 085-35-00W,21-43-00N 086-42-00W,22-16-00N 088-32-00W,22-30-00N 088-38-00W,23-26-00N 091-10-00W,23-18-00N 091-45-00W,24-06-00N 094-21-00W,25-38-00N 096-49-00W AND25-48-00N 097-05-00W.2. PRIMARY AND BACKUP LAUNCH DAY HAZARD PERIODS INCLUDE:16/2245Z JUL 26 TO 17/0056Z JUL 2617/2245Z JUL 26 TO 18/0056Z JUL 2618/2245Z JUL 26 TO 19/0056Z JUL 2619/2245Z JUL 26 TO 20/0056Z JUL 2620/2245Z JUL 26 TO 21/0056Z JUL 2621/2245Z JUL 26 TO 22/0056Z JUL 2622/2245Z JUL 26 TO 23/0056Z JUL 26 3. NAVIGATION HAZARDS WITHIN THE HAZARD AREAS MAY INCLUDE FREE FALLING DEBRIS AND/OR DESCENDING VEHICLES OR VEHICLE COMPONENTS UNDER VARIOUS MEANS OF CONTROL. FREE FALLING ROCKET LAUNCHING COMPONENTS WILL LAND WITHIN THE HIGH RISK HAZARD AREA. MARINERS SHOULD AVOID WATERS WITHIN THE DEFINED HAZARD AREAS DURING THE SCHEDULED LAUNCH WINDOW. THE HIGH RISK HAZARD AREA SHOULD BE AVOIDED THREE HOURS PRIOR TO THE EARLIEST LAUNCH TO ENSURE RANGE CLEARANCE. FOR ADDITIONAL INFORMATION, CONTACT THE U.S. COAST GUARD SECTOR CORPUS CHRISTI COMMAND CENTER AT (800) 874-2143, OR ACCESS: WWW.NAVCEN.USCG.GOV/MSI CANCEL AT//230156Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1097,14 +1097,14 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K15" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1114,27 +1114,27 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46213.22780092592</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0043-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1146,14 +1146,14 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>110</v>
+        <v>10.3</v>
       </c>
       <c r="K16" t="n">
-        <v>118</v>
+        <v>10.3</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1163,27 +1163,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>OUACHITA RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46212.59893518518</v>
+        <v>46213.22780092592</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0042-26</t>
+          <t>SEC LMR BNM 0043-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1202,7 +1202,7 @@
         <v>110</v>
       </c>
       <c r="K17" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
@@ -1212,27 +1212,27 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>OUACHITA RIVER</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
+          <t>1.The Coast Guard is establishing temporary special local regulation for Ouachita River MM 110-118 from 7 a.m. through 1 p.m. on July 11th, 2026. This is to ensure the safety of life and property during a permitted marine event.2.No vessels may enter or remain within this area unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//111300 JUL 26//. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46210.47041666666</v>
+        <v>46212.59893518518</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0075-26</t>
+          <t>SEC LMR BNM 0042-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1242,9 +1242,17 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>110</v>
+      </c>
+      <c r="K18" t="n">
+        <v>117</v>
+      </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
@@ -1253,27 +1261,27 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
+          <t>1. MARINERS BE ADVISED OF MISSING BUOYS BETWEEN ARK MM 110-117. EXERCISE CAUTION DURING TRANSIT.2. REPORT FURTHER DISCREPANCIES TO THE U.S. COAST GUARD VIA TELEPHONE AT 866-360-3386. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46209.69443287037</v>
+        <v>46210.47041666666</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0074-26</t>
+          <t>CGD-H BNM 0075-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1294,27 +1302,27 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
+          <t>AN ORANGE AND WHITE BUOY WITH A FLASHING 2.5 SECONDWHITE LIGHT HAS BEEN TEMPORARILY ESTABLISHED IN SOUTHPASS AREA, BLOCK 60, IN APPROX POSITION 29-03-18.904N 088-58-13.511W. THE BUOY IS MARKING THE LOWER JACKET AND SUBSEA HAZARDS WITHIN 2000 FT OF PLATFORM DEMOLITION SITES.MARINERS SHOULD AVOID THE AREA.CANCEL AT//290500Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46208.56896990741</v>
+        <v>46209.69443287037</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0040-26</t>
+          <t>CGD-H BNM 0074-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1333,25 +1341,29 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
+          <t>ON 08JUL2026, FROM 1300Z TO 2000Z, THE U.S. NAVY WILL CONDUCT UNDERWATER DETONATIONS IN THE GULF OF AMERICA, IN APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. THE BACK-UP DATE IS SCHEDULED FOR 09JUL2026. MARINERS SHOULD MAINTAINA 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//092100Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46207.88481481482</v>
+        <v>46208.56896990741</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0041-26</t>
+          <t>SEC LMR BNM 0040-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1374,14 +1386,14 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0040-26 DTG 191905Z JUN 26</t>
         </is>
       </c>
       <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46203.47113425926</v>
+        <v>46207.88481481482</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
@@ -1407,38 +1419,30 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//. BT</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46202.62762731482</v>
+        <v>46203.47113425926</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0073-26</t>
+          <t>SEC LMR BNM 0041-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>other_NA</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1454,40 +1458,36 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
+          <t>1.The Coast Guard is establishing temporary safety zone on the LMR between mile markers 735.5 - 736.5 to ensure the safety of life and property during an overwater drone flight on July 3rd, 2026. The safety zone will be in effect from 8 p.m. through 10 p.m.2.No vessels may enter or remain within this zone unless specifically authorized by the Captain of the Port Sector Lower Mississippi River. Vessels may contact Coast Guard Western Rivers Command Center on VHF-FM channel 16 for further information.3.Cancel at TIME//032200 JUL 26//.</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46198.35914351852</v>
+        <v>46202.62762731482</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0073-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>cancellation</t>
+          <t>other_NA</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1501,11 +1501,15 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>ON 30JUN2026 THROUGH 02JUL2026, FROM 1100Z TO 2300Z, THE U.S. NAVY WILL CONDUCT DAILY LIVE ORDNANCE OPERATIONS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-06-28.32N 085-25-42.36W, 29-06-08.16N 084-58-54.12W, 28-43-04.80N 084-58-54.12W AND 28-43-24.66N 085-25-42.36W.MARINERS SHOULD MAINTAIN A 1-MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA.CANCEL AT//022359Z JUL 26// BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1516,40 +1520,32 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46190.37179398148</v>
+        <v>46198.35914351852</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0069-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
-        </is>
-      </c>
+          <t>cancellation</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="n">
-        <v>28.8597396564073</v>
-      </c>
-      <c r="M25" t="n">
-        <v>-94.1676102718865</v>
-      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
@@ -1558,7 +1554,7 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0039-26 DTG 131850Z JUN 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1569,67 +1565,49 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46190.37179398148</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0069-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dredging</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Approach of potential tropical storm in Gulf region: Texas, Louisiana</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
-        <v>35.07917</v>
+        <v>28.8597396564073</v>
       </c>
       <c r="M26" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N26" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>46195</v>
-      </c>
+        <v>-94.1676102718865</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>WITH THE APPROACH OF POTENTIAL TROPICAL CYCLONE ONE, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//181700Z JUN 26// BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1640,53 +1618,67 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K27" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1697,61 +1689,53 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K28" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O28" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1762,57 +1746,61 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K29" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1823,37 +1811,37 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K30" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
@@ -1863,17 +1851,17 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1884,11 +1872,9 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
@@ -1897,48 +1883,46 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K31" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1949,23 +1933,25 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B32" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1976,30 +1962,32 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K32" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2010,65 +1998,57 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N33" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O33" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J33" t="n">
+        <v>603</v>
+      </c>
+      <c r="K33" t="n">
+        <v>603</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2079,12 +2059,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B34" t="inlineStr"/>
-      <c r="C34" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>N</t>
@@ -2092,48 +2070,54 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>585</v>
-      </c>
-      <c r="K34" t="n">
-        <v>869</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M34" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N34" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2144,11 +2128,11 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2157,7 +2141,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2173,7 +2157,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K35" t="n">
         <v>869</v>
@@ -2181,7 +2165,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
@@ -2191,14 +2175,14 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2209,11 +2193,11 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2222,7 +2206,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2241,17 +2225,17 @@
         <v>303</v>
       </c>
       <c r="K36" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -2263,7 +2247,7 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2274,11 +2258,11 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2287,7 +2271,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2311,7 +2295,7 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
@@ -2328,7 +2312,7 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2339,10 +2323,12 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>N</t>
@@ -2350,54 +2336,48 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M38" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J38" t="n">
+        <v>303</v>
+      </c>
+      <c r="K38" t="n">
+        <v>585</v>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2408,57 +2388,65 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K39" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2469,25 +2457,23 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2498,32 +2484,30 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K40" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2534,11 +2518,11 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2547,7 +2531,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2571,12 +2555,12 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -2588,10 +2572,75 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>303</v>
+      </c>
+      <c r="K42" t="n">
+        <v>869</v>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-12: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,178 +541,174 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.49533564815</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0083-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>785</v>
-      </c>
-      <c r="K2" t="n">
-        <v>785</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K3" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K4" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="N4" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -726,102 +722,82 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K6" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -831,17 +807,9 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>857</v>
-      </c>
-      <c r="K7" t="n">
-        <v>867</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -850,13 +818,13 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -867,161 +835,155 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K8" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="N8" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M9" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J9" t="n">
+        <v>857</v>
+      </c>
+      <c r="K9" t="n">
+        <v>867</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K10" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
@@ -1029,28 +991,30 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B11" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
@@ -1059,50 +1023,54 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K11" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M11" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N11" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1113,7 +1081,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
@@ -1124,7 +1092,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1140,10 +1108,10 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K12" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1151,19 +1119,15 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1174,7 +1138,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
@@ -1185,12 +1149,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1201,30 +1165,34 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K13" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="N13" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1235,25 +1203,23 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
@@ -1264,32 +1230,30 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K14" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1300,37 +1264,37 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K15" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1340,17 +1304,17 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1361,9 +1325,11 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B16" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
@@ -1372,54 +1338,48 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J16" t="n">
+        <v>303</v>
+      </c>
+      <c r="K16" t="n">
+        <v>869</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1430,25 +1390,23 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1459,32 +1417,30 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K17" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1495,12 +1451,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B18" t="inlineStr"/>
-      <c r="C18" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>N</t>
@@ -1508,48 +1462,54 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>303</v>
-      </c>
-      <c r="K18" t="n">
-        <v>869</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M18" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N18" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1560,11 +1520,11 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1573,7 +1533,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1589,32 +1549,32 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K19" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1625,11 +1585,11 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1638,7 +1598,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1657,17 +1617,17 @@
         <v>303</v>
       </c>
       <c r="K20" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -1679,7 +1639,7 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1690,10 +1650,12 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1701,54 +1663,48 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M21" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J21" t="n">
+        <v>303</v>
+      </c>
+      <c r="K21" t="n">
+        <v>585</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1759,23 +1715,25 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1786,30 +1744,32 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K22" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1820,12 +1780,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>N</t>
@@ -1833,48 +1791,54 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>303</v>
-      </c>
-      <c r="K23" t="n">
-        <v>869</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1885,25 +1849,23 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1914,35 +1876,163 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K24" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" s="2" t="n">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>303</v>
+      </c>
+      <c r="K25" t="n">
+        <v>869</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>869</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr">
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-13: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46245.49533564815</v>
+        <v>46246.68484953704</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0083-26</t>
+          <t>CGD-H BNM 0084-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -575,21 +575,21 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+          <t>ON 14AUG2026, FROM 1900Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//142200Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46245.49533564815</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0083-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -599,17 +599,9 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K3" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,115 +610,123 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K4" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>785</v>
+      </c>
+      <c r="K5" t="n">
+        <v>785</v>
+      </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="N5" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -737,67 +737,55 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K6" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -807,9 +795,17 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K7" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -818,13 +814,13 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -835,136 +831,128 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>849</v>
-      </c>
-      <c r="K8" t="n">
-        <v>849</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K9" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="N9" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -976,14 +964,14 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K10" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
@@ -993,13 +981,13 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1010,124 +998,120 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K11" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B12" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K12" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M12" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1138,61 +1122,53 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K13" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1203,57 +1179,61 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K14" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="N14" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1264,37 +1244,37 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K15" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1304,17 +1284,17 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1325,11 +1305,9 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
@@ -1338,48 +1316,46 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K16" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1390,23 +1366,25 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B17" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1417,30 +1395,32 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K17" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
+      <c r="N17" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1451,65 +1431,57 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M18" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J18" t="n">
+        <v>603</v>
+      </c>
+      <c r="K18" t="n">
+        <v>603</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1520,12 +1492,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B19" t="inlineStr"/>
-      <c r="C19" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>N</t>
@@ -1533,48 +1503,54 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>585</v>
-      </c>
-      <c r="K19" t="n">
-        <v>869</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N19" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1585,11 +1561,11 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1598,7 +1574,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1614,7 +1590,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K20" t="n">
         <v>869</v>
@@ -1622,7 +1598,7 @@
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
@@ -1632,14 +1608,14 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1650,11 +1626,11 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1663,7 +1639,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1682,17 +1658,17 @@
         <v>303</v>
       </c>
       <c r="K21" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -1704,7 +1680,7 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1715,11 +1691,11 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1728,7 +1704,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1752,7 +1728,7 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
@@ -1769,7 +1745,7 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1780,10 +1756,12 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>N</t>
@@ -1791,54 +1769,48 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M23" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J23" t="n">
+        <v>303</v>
+      </c>
+      <c r="K23" t="n">
+        <v>585</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1849,57 +1821,65 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K24" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M24" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1910,25 +1890,23 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1939,32 +1917,30 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K25" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1975,11 +1951,11 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1988,7 +1964,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2012,12 +1988,12 @@
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2029,10 +2005,75 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>303</v>
+      </c>
+      <c r="K27" t="n">
+        <v>869</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-15: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46246.68484953704</v>
+        <v>46248.60054398148</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0084-26</t>
+          <t>CGD-H BNM 0089-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -569,27 +569,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 14AUG2026, FROM 1900Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//142200Z AUG 26// BT</t>
+          <t>FROM 15AUG2026 TO 04SEP2026, THE M/V SEVAN LOUISIANA WILL CONDUCT DIVING OPERATIONS IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-50-42N 090-05-24W. MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//050500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46245.49533564815</v>
+        <v>46248.60001157408</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0083-26</t>
+          <t>CGD-H BNM 0088-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -610,27 +610,27 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+          <t>BETWEEN 17AUG2026 AND 31AUG2026, THE U.S. NAVY WILL CONDUCT DAILY SURFACE TESTS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-55-04.06N 086-10-03.44W,29-55-04.49N 086-11-12.50W,29-54-04.33N 086-11-12.99W AND29-54-03.90N 086-10-03.94W.MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACHFROM THE OPERATING AREA.CANCEL AT//010500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46248.59320601852</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -640,17 +640,9 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K4" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -659,97 +651,73 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 29-06-54N 085-00-43W,28-08-03N 083-56-46W,27-50-04N 084-18-00W AND28-48-46N 085-21-59W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46248.58787037037</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>785</v>
-      </c>
-      <c r="K5" t="n">
-        <v>785</v>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-23-29N 086-49-21W,30-24-18N 086-48-23W,30-24-09N 086-43-22W,30-21-57N 086-32-55W,30-12-09N 086-27-17W,30-05-20N 086-35-25W,30-08-28N 086-46-42W AND30-19-30N 086-49-47W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46248.58724537037</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>CGD-H BNM 0085-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -763,29 +731,29 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>FL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>FROM 1300Z TO 2000Z, ON 17AUG2026, BACKUP DATE 18AUG2026,THE U.S. NAVY WILL CONDUCT ORDINANCE OPERATIONS IN THE GULF OF AMERICA NEAR APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. MARINERS SHOULD MAINTAIN A 1 MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL SUPPORT CRAFT. CANCEL AT//182100Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46246.68484953704</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>CGD-H BNM 0084-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -795,17 +763,9 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K7" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -814,31 +774,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 14AUG2026, FROM 1900Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//142200Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46245.49533564815</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>CGD-H BNM 0083-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -859,381 +815,331 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>849</v>
+        <v>435.8</v>
       </c>
       <c r="K9" t="n">
-        <v>849</v>
+        <v>435.8</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>857</v>
+        <v>785</v>
       </c>
       <c r="K10" t="n">
-        <v>867</v>
+        <v>785</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K11" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46239.68305555556</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K12" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K13" t="n">
-        <v>777.7</v>
-      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>125.4</v>
+        <v>849</v>
       </c>
       <c r="K14" t="n">
-        <v>155.9</v>
+        <v>849</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>46146</v>
+        <v>46234</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>46188</v>
+        <v>46243</v>
       </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1244,23 +1150,19 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1271,10 +1173,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>686</v>
+        <v>857</v>
       </c>
       <c r="K15" t="n">
-        <v>686</v>
+        <v>867</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1284,44 +1186,36 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1332,10 +1226,10 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>348.7</v>
+        <v>10.3</v>
       </c>
       <c r="K16" t="n">
-        <v>348.7</v>
+        <v>10.3</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1345,31 +1239,27 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>"Possible shoaling," transit area with caution</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46065.67140046296</v>
+        <v>46186.8905787037</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>46070</v>
+        <v>46199</v>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
@@ -1379,48 +1269,54 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>303</v>
-      </c>
-      <c r="K17" t="n">
-        <v>869</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+        <v>46188</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1431,7 +1327,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1442,7 +1338,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1458,10 +1354,10 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>603</v>
+        <v>777.7</v>
       </c>
       <c r="K18" t="n">
-        <v>603</v>
+        <v>777.7</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
@@ -1469,11 +1365,7 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr">
         <is>
           <t>Proceed with caution</t>
@@ -1481,7 +1373,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1492,7 +1384,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1503,54 +1395,50 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>125.4</v>
+      </c>
+      <c r="K19" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>46062</v>
+        <v>46146</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>46065</v>
+        <v>46188</v>
       </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1561,25 +1449,23 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1590,32 +1476,30 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>585</v>
+        <v>686</v>
       </c>
       <c r="K20" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1626,12 +1510,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1639,48 +1521,46 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K21" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1691,12 +1571,12 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46050.44465277778</v>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" s="2" t="n">
-        <v>46052</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>N</t>
@@ -1704,7 +1584,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1723,17 +1603,17 @@
         <v>303</v>
       </c>
       <c r="K22" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>46050</v>
+        <v>46068</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1745,7 +1625,7 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1756,25 +1636,23 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1785,32 +1663,30 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K23" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1821,7 +1697,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
@@ -1832,7 +1708,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1854,32 +1730,32 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
-        <v>35.0859560963022</v>
+        <v>35.085769</v>
       </c>
       <c r="M24" t="n">
-        <v>-90.10785143484679</v>
+        <v>-90.10947400000001</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46062</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>46044</v>
+        <v>46065</v>
       </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
+          <t>Amrize Dock on Mckellar Lake</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1890,23 +1766,25 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1917,30 +1795,32 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="K25" t="n">
-        <v>538.7</v>
+        <v>869</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1951,11 +1831,11 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="2" t="n">
-        <v>46045</v>
+        <v>46061</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1964,7 +1844,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1988,7 +1868,7 @@
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
@@ -2005,7 +1885,7 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2016,11 +1896,11 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="2" t="n">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2029,7 +1909,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2048,17 +1928,17 @@
         <v>303</v>
       </c>
       <c r="K27" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>46034</v>
+        <v>46050</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2070,10 +1950,335 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>303</v>
+      </c>
+      <c r="K28" t="n">
+        <v>585</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M29" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K30" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>303</v>
+      </c>
+      <c r="K31" t="n">
+        <v>869</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>303</v>
+      </c>
+      <c r="K32" t="n">
+        <v>869</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-18: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,26 +541,34 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46248.60054398148</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0089-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>736</v>
+      </c>
+      <c r="K2" t="n">
+        <v>736</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,27 +577,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>LA - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>FROM 15AUG2026 TO 04SEP2026, THE M/V SEVAN LOUISIANA WILL CONDUCT DIVING OPERATIONS IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-50-42N 090-05-24W. MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//050500Z SEP 26// BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46248.60001157408</v>
+        <v>46251.58429398148</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0088-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -608,29 +616,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>FL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>BETWEEN 17AUG2026 AND 31AUG2026, THE U.S. NAVY WILL CONDUCT DAILY SURFACE TESTS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-55-04.06N 086-10-03.44W,29-55-04.49N 086-11-12.50W,29-54-04.33N 086-11-12.99W AND29-54-03.90N 086-10-03.94W.MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACHFROM THE OPERATING AREA.CANCEL AT//010500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0051-26 DTG 101204Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46248.59320601852</v>
+        <v>46251.42490740741</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0090-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -651,27 +655,27 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 29-06-54N 085-00-43W,28-08-03N 083-56-46W,27-50-04N 084-18-00W AND28-48-46N 085-21-59W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
+          <t>ON 18AUG2026, FROM 1600Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//182200Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46248.58787037037</v>
+        <v>46248.60054398148</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0089-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -692,27 +696,27 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>FL - GULF OF AMERICA</t>
+          <t>LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-23-29N 086-49-21W,30-24-18N 086-48-23W,30-24-09N 086-43-22W,30-21-57N 086-32-55W,30-12-09N 086-27-17W,30-05-20N 086-35-25W,30-08-28N 086-46-42W AND30-19-30N 086-49-47W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
+          <t>FROM 15AUG2026 TO 04SEP2026, THE M/V SEVAN LOUISIANA WILL CONDUCT DIVING OPERATIONS IN THE GULF OF AMERICA, GRAND ISLE AREA, IN APPROXIMATE POSITION 28-50-42N 090-05-24W. MARINERS SHOULD MAINTAIN A WIDE BERTH FROM THE DIVE VESSEL. CANCEL AT//050500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46248.58724537037</v>
+        <v>46248.60001157408</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0085-26</t>
+          <t>CGD-H BNM 0088-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -739,21 +743,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>FROM 1300Z TO 2000Z, ON 17AUG2026, BACKUP DATE 18AUG2026,THE U.S. NAVY WILL CONDUCT ORDINANCE OPERATIONS IN THE GULF OF AMERICA NEAR APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. MARINERS SHOULD MAINTAIN A 1 MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL SUPPORT CRAFT. CANCEL AT//182100Z AUG 26// BT</t>
+          <t>BETWEEN 17AUG2026 AND 31AUG2026, THE U.S. NAVY WILL CONDUCT DAILY SURFACE TESTS IN THE GULF OF AMERICA, IN AN AREA BOUND BY APPROXIMATE POSITIONS: 29-55-04.06N 086-10-03.44W,29-55-04.49N 086-11-12.50W,29-54-04.33N 086-11-12.99W AND29-54-03.90N 086-10-03.94W.MARINERS SHOULD MAINTAIN A 1 NM CLOSEST POINT OF APPROACHFROM THE OPERATING AREA.CANCEL AT//010500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46246.68484953704</v>
+        <v>46248.59320601852</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0084-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -774,27 +778,27 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>ON 14AUG2026, FROM 1900Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//142200Z AUG 26// BT</t>
+          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 29-06-54N 085-00-43W,28-08-03N 083-56-46W,27-50-04N 084-18-00W AND28-48-46N 085-21-59W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46245.49533564815</v>
+        <v>46248.58787037037</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0083-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -815,27 +819,27 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+          <t>THE USAF WILL CONDUCT DAILY MUNITION LAUNCHES OFF SANTA ROSA ISLAND INTO THE GULF OF AMERICA. THE HAZARD AREA WILL BE ACTIVE 17AUG2026, FROM 1600Z TO 2130Z, AND 18AUG2026 TO 28AUG2026, FROM 1300Z TO 1630Z AND 1900Z TO 2130Z. THE HAZARD AREA WILL BE BOUND BY APPROXIMATE POSITIONS: 30-23-29N 086-49-21W,30-24-18N 086-48-23W,30-24-09N 086-43-22W,30-21-57N 086-32-55W,30-12-09N 086-27-17W,30-05-20N 086-35-25W,30-08-28N 086-46-42W AND30-19-30N 086-49-47W.MARINERS ARE URGED TO AVOID THE HAZARD AREA.CANCEL AT//282230Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46248.58724537037</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0085-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -845,17 +849,9 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K9" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -864,97 +860,73 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>FL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>FROM 1300Z TO 2000Z, ON 17AUG2026, BACKUP DATE 18AUG2026,THE U.S. NAVY WILL CONDUCT ORDINANCE OPERATIONS IN THE GULF OF AMERICA NEAR APPROXIMATE POSITION 30-19-05.76N 086-33-04.80W. MARINERS SHOULD MAINTAIN A 1 MILE CLOSEST POINT OF APPROACH FROM THE OPERATING AREA AND ALL NAVAL SUPPORT CRAFT. CANCEL AT//182100Z AUG 26// BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46246.68484953704</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>CGD-H BNM 0084-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>785</v>
-      </c>
-      <c r="K10" t="n">
-        <v>785</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 14AUG2026, FROM 1900Z TO 2100Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//142200Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.49533564815</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>CGD-H BNM 0083-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -968,29 +940,29 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>AL - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 14AUG2026, FROM 0045Z TO 0400Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 10,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//140500Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1002,14 +974,14 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="K12" t="n">
-        <v>325.2</v>
+        <v>435.8</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1019,77 +991,89 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>785</v>
+      </c>
+      <c r="K13" t="n">
+        <v>785</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="N13" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0046-26</t>
@@ -1097,49 +1081,25 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>849</v>
-      </c>
-      <c r="K14" t="n">
-        <v>849</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1150,14 +1110,14 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1169,14 +1129,14 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>857</v>
+        <v>325.2</v>
       </c>
       <c r="K15" t="n">
-        <v>867</v>
+        <v>325.2</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1186,13 +1146,13 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1203,14 +1163,14 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1220,17 +1180,9 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="K16" t="n">
-        <v>10.3</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1239,13 +1191,13 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1256,20 +1208,18 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46234.89293981482</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1288,35 +1238,35 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M17" t="n">
-        <v>-90.17319999999999</v>
-      </c>
+      <c r="J17" t="n">
+        <v>849</v>
+      </c>
+      <c r="K17" t="n">
+        <v>849</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>46188</v>
+        <v>46234</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>46195</v>
+        <v>46243</v>
       </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1327,23 +1277,19 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1354,10 +1300,10 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>777.7</v>
+        <v>857</v>
       </c>
       <c r="K18" t="n">
-        <v>777.7</v>
+        <v>867</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
@@ -1365,42 +1311,38 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1411,95 +1353,97 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>125.4</v>
+        <v>10.3</v>
       </c>
       <c r="K19" t="n">
-        <v>155.9</v>
+        <v>10.3</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46119.48518518519</v>
-      </c>
-      <c r="B20" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>686</v>
-      </c>
-      <c r="K20" t="n">
-        <v>686</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1510,37 +1454,37 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="K21" t="n">
-        <v>348.7</v>
+        <v>777.7</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
@@ -1548,19 +1492,15 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1571,11 +1511,9 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46146.4284375</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
@@ -1584,48 +1522,50 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>303</v>
+        <v>125.4</v>
       </c>
       <c r="K22" t="n">
-        <v>869</v>
+        <v>155.9</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+        <v>46146</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1636,7 +1576,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
@@ -1647,7 +1587,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1663,10 +1603,10 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="K23" t="n">
-        <v>603</v>
+        <v>686</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
@@ -1676,17 +1616,17 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1697,7 +1637,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
@@ -1708,54 +1648,46 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M24" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N24" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>46065</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>348.7</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1766,12 +1698,12 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46058.58436342593</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" s="2" t="n">
-        <v>46068</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>N</t>
@@ -1779,7 +1711,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1795,7 +1727,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>585</v>
+        <v>303</v>
       </c>
       <c r="K25" t="n">
         <v>869</v>
@@ -1803,7 +1735,7 @@
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
@@ -1813,14 +1745,14 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>10'6" draft, 6 barges wide</t>
+          <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1831,25 +1763,23 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1860,32 +1790,30 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>303</v>
+        <v>603</v>
       </c>
       <c r="K26" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1896,12 +1824,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>N</t>
@@ -1909,48 +1835,54 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>303</v>
-      </c>
-      <c r="K27" t="n">
-        <v>585</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N27" s="2" t="n">
-        <v>46050</v>
-      </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1961,11 +1893,11 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="2" t="n">
-        <v>46050</v>
+        <v>46068</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1974,7 +1906,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1990,32 +1922,32 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K28" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>46045</v>
+        <v>46061</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2026,10 +1958,12 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" s="2" t="n">
+        <v>46061</v>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>N</t>
@@ -2037,54 +1971,48 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M29" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J29" t="n">
+        <v>303</v>
+      </c>
+      <c r="K29" t="n">
+        <v>869</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O29" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46052</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2095,23 +2023,25 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -2122,30 +2052,32 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K30" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -2156,11 +2088,11 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2169,7 +2101,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2188,17 +2120,17 @@
         <v>303</v>
       </c>
       <c r="K31" t="n">
-        <v>869</v>
+        <v>585</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2210,7 +2142,7 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -2221,64 +2153,259 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M32" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K33" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>303</v>
+      </c>
+      <c r="K34" t="n">
+        <v>869</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
         <v>46033.86975694444</v>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" s="2" t="n">
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" s="2" t="n">
         <v>46037</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>SEC LMR BNM 0106-26</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J32" t="n">
+      <c r="J35" t="n">
         <v>303</v>
       </c>
-      <c r="K32" t="n">
+      <c r="K35" t="n">
         <v>869</v>
       </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr">
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-22: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -558,9 +558,17 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K2" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,116 +577,104 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>736</v>
-      </c>
-      <c r="K3" t="n">
-        <v>736</v>
-      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K4" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="N4" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
@@ -689,113 +685,125 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K5" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>785</v>
+      </c>
+      <c r="K6" t="n">
+        <v>785</v>
+      </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+      <c r="N6" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -806,67 +814,55 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K7" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -876,9 +872,17 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
@@ -887,13 +891,13 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -904,136 +908,128 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>849</v>
-      </c>
-      <c r="K9" t="n">
-        <v>849</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K10" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O10" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1045,14 +1041,14 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K11" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
@@ -1062,13 +1058,13 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1079,124 +1075,120 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B13" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K13" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M13" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1207,61 +1199,53 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K14" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1272,57 +1256,61 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K15" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="N15" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1333,37 +1321,37 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K16" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
@@ -1373,17 +1361,17 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1394,11 +1382,9 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
@@ -1407,48 +1393,46 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K17" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1459,23 +1443,25 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B18" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1486,30 +1472,32 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K18" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1520,65 +1508,57 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M19" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N19" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J19" t="n">
+        <v>603</v>
+      </c>
+      <c r="K19" t="n">
+        <v>603</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1589,12 +1569,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>N</t>
@@ -1602,48 +1580,54 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>585</v>
-      </c>
-      <c r="K20" t="n">
-        <v>869</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1654,11 +1638,11 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1667,7 +1651,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1683,7 +1667,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K21" t="n">
         <v>869</v>
@@ -1691,7 +1675,7 @@
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
@@ -1701,14 +1685,14 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1719,11 +1703,11 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1732,7 +1716,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1751,17 +1735,17 @@
         <v>303</v>
       </c>
       <c r="K22" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1773,7 +1757,7 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1784,11 +1768,11 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1797,7 +1781,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1821,7 +1805,7 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
@@ -1838,7 +1822,7 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1849,10 +1833,12 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>N</t>
@@ -1860,54 +1846,48 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M24" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J24" t="n">
+        <v>303</v>
+      </c>
+      <c r="K24" t="n">
+        <v>585</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1918,57 +1898,65 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K25" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M25" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1979,25 +1967,23 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -2008,32 +1994,30 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K26" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N26" t="inlineStr"/>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2044,11 +2028,11 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2057,7 +2041,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2081,12 +2065,12 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2098,10 +2082,75 @@
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>303</v>
+      </c>
+      <c r="K28" t="n">
+        <v>869</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-24: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -558,46 +558,34 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K2" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -607,9 +595,17 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K3" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -618,116 +614,104 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>736</v>
-      </c>
-      <c r="K4" t="n">
-        <v>736</v>
-      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K5" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="N5" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
@@ -738,113 +722,125 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K6" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>785</v>
+      </c>
+      <c r="K7" t="n">
+        <v>785</v>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="N7" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -855,67 +851,55 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K8" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -925,9 +909,17 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K9" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -936,13 +928,13 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -953,136 +945,128 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>849</v>
-      </c>
-      <c r="K10" t="n">
-        <v>849</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K11" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+      <c r="N11" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1094,14 +1078,14 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K12" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
@@ -1111,13 +1095,13 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1128,124 +1112,120 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K14" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M14" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1256,61 +1236,53 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K15" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -1321,57 +1293,61 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K16" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="N16" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1382,37 +1358,37 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K17" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
@@ -1422,17 +1398,17 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1443,11 +1419,9 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
@@ -1456,48 +1430,46 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K18" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1508,23 +1480,25 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B19" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1535,30 +1509,32 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K19" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1569,65 +1545,57 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M20" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N20" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J20" t="n">
+        <v>603</v>
+      </c>
+      <c r="K20" t="n">
+        <v>603</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1638,12 +1606,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B21" t="inlineStr"/>
-      <c r="C21" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1651,48 +1617,54 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>585</v>
-      </c>
-      <c r="K21" t="n">
-        <v>869</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N21" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1703,11 +1675,11 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1716,7 +1688,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1732,7 +1704,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K22" t="n">
         <v>869</v>
@@ -1740,7 +1712,7 @@
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
@@ -1750,14 +1722,14 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1768,11 +1740,11 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1781,7 +1753,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1800,17 +1772,17 @@
         <v>303</v>
       </c>
       <c r="K23" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -1822,7 +1794,7 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1833,11 +1805,11 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1846,7 +1818,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1870,7 +1842,7 @@
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
@@ -1887,7 +1859,7 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1898,10 +1870,12 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>N</t>
@@ -1909,54 +1883,48 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M25" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J25" t="n">
+        <v>303</v>
+      </c>
+      <c r="K25" t="n">
+        <v>585</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1967,57 +1935,65 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K26" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2028,25 +2004,23 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -2057,32 +2031,30 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K27" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2093,11 +2065,11 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2106,7 +2078,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2130,12 +2102,12 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2147,10 +2119,75 @@
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>303</v>
+      </c>
+      <c r="K29" t="n">
+        <v>869</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-25: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -571,21 +571,21 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -595,46 +595,34 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K3" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -653,65 +641,49 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K5" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O5" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
@@ -722,25 +694,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -750,17 +718,9 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K6" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -769,24 +729,20 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
@@ -797,7 +753,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -817,30 +773,30 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K7" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -851,113 +807,137 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K8" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K9" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="N9" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -971,102 +951,82 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K11" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1076,17 +1036,9 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>857</v>
-      </c>
-      <c r="K12" t="n">
-        <v>867</v>
-      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -1095,13 +1047,13 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1112,161 +1064,155 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K13" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="N13" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O13" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M14" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J14" t="n">
+        <v>857</v>
+      </c>
+      <c r="K14" t="n">
+        <v>867</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K15" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1274,28 +1220,30 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B16" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
@@ -1304,50 +1252,54 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K16" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M16" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N16" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -1358,7 +1310,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
@@ -1369,7 +1321,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1385,10 +1337,10 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K17" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
@@ -1396,19 +1348,15 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1419,7 +1367,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
@@ -1430,12 +1378,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -1446,30 +1394,34 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K18" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="N18" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -1480,25 +1432,23 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1509,32 +1459,30 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K19" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1545,37 +1493,37 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K20" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
@@ -1585,17 +1533,17 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1606,9 +1554,11 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B21" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
@@ -1617,54 +1567,48 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M21" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J21" t="n">
+        <v>303</v>
+      </c>
+      <c r="K21" t="n">
+        <v>869</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1675,25 +1619,23 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B22" t="inlineStr"/>
-      <c r="C22" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1704,32 +1646,30 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K22" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1740,12 +1680,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B23" t="inlineStr"/>
-      <c r="C23" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>N</t>
@@ -1753,48 +1691,54 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>303</v>
-      </c>
-      <c r="K23" t="n">
-        <v>869</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1805,11 +1749,11 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1818,7 +1762,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1834,32 +1778,32 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K24" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -1870,11 +1814,11 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1883,7 +1827,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1902,17 +1846,17 @@
         <v>303</v>
       </c>
       <c r="K25" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -1924,7 +1868,7 @@
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1935,10 +1879,12 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>N</t>
@@ -1946,54 +1892,48 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M26" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J26" t="n">
+        <v>303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>585</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -2004,23 +1944,25 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -2031,30 +1973,32 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K27" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2065,12 +2009,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>N</t>
@@ -2078,48 +2020,54 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>303</v>
-      </c>
-      <c r="K28" t="n">
-        <v>869</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M28" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N28" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2130,25 +2078,23 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B29" t="inlineStr"/>
-      <c r="C29" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
@@ -2159,35 +2105,163 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K29" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" s="2" t="n">
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>303</v>
+      </c>
+      <c r="K30" t="n">
+        <v>869</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>303</v>
+      </c>
+      <c r="K31" t="n">
+        <v>869</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr">
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-08-31: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -567,25 +567,29 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -608,21 +612,21 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -645,21 +649,21 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -669,46 +673,34 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K5" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -727,94 +719,62 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>736</v>
-      </c>
-      <c r="K7" t="n">
-        <v>736</v>
-      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -824,120 +784,76 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K8" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>785</v>
-      </c>
-      <c r="K9" t="n">
-        <v>785</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Osceola Harbor</t>
-        </is>
-      </c>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -955,25 +871,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -983,17 +895,9 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K11" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -1002,31 +906,27 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1045,102 +945,62 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>849</v>
-      </c>
-      <c r="K13" t="n">
-        <v>849</v>
-      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1150,50 +1010,34 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>857</v>
-      </c>
-      <c r="K14" t="n">
-        <v>867</v>
-      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1205,14 +1049,14 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>10.3</v>
+        <v>661.7</v>
       </c>
       <c r="K15" t="n">
-        <v>10.3</v>
+        <v>661.7</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
@@ -1222,95 +1066,61 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46253.46241898148</v>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M16" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N16" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O16" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>AL - GULF OF AMERICA</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
@@ -1321,42 +1131,50 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>777.7</v>
+        <v>736</v>
       </c>
       <c r="K17" t="n">
-        <v>777.7</v>
+        <v>736</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
+      <c r="N17" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -1367,72 +1185,60 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>125.4</v>
+        <v>435.8</v>
       </c>
       <c r="K18" t="n">
-        <v>155.9</v>
+        <v>435.8</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
@@ -1443,46 +1249,50 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>686</v>
+        <v>785</v>
       </c>
       <c r="K19" t="n">
-        <v>686</v>
+        <v>785</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="N19" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
-        </is>
-      </c>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -1493,57 +1303,37 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>348.7</v>
-      </c>
-      <c r="K20" t="n">
-        <v>348.7</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>Mid channel</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>"Possible shoaling," transit area with caution</t>
-        </is>
-      </c>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1554,103 +1344,79 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46239.68305555556</v>
+      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>303</v>
+        <v>325.2</v>
       </c>
       <c r="K21" t="n">
-        <v>869</v>
+        <v>325.2</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>603</v>
-      </c>
-      <c r="K22" t="n">
-        <v>603</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -1659,39 +1425,35 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1710,35 +1472,35 @@
           <t>LMR</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M23" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J23" t="n">
+        <v>849</v>
+      </c>
+      <c r="K23" t="n">
+        <v>849</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46062</v>
+        <v>46234</v>
       </c>
       <c r="O23" s="2" t="n">
-        <v>46065</v>
+        <v>46243</v>
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1749,25 +1511,19 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B24" t="inlineStr"/>
-      <c r="C24" s="2" t="n">
-        <v>46068</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1778,113 +1534,95 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>585</v>
+        <v>857</v>
       </c>
       <c r="K24" t="n">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B25" t="inlineStr"/>
-      <c r="C25" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>303</v>
+        <v>10.3</v>
       </c>
       <c r="K25" t="n">
-        <v>869</v>
+        <v>10.3</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46052</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46050.44465277778</v>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" s="2" t="n">
-        <v>46052</v>
-      </c>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>N</t>
@@ -1892,48 +1630,54 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>303</v>
-      </c>
-      <c r="K26" t="n">
-        <v>585</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M26" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N26" s="2" t="n">
-        <v>46050</v>
-      </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+        <v>46188</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1944,25 +1688,23 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" s="2" t="n">
-        <v>46050</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1973,32 +1715,26 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>303</v>
+        <v>777.7</v>
       </c>
       <c r="K27" t="n">
-        <v>585</v>
+        <v>777.7</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -2009,7 +1745,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
@@ -2020,54 +1756,50 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M28" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>125.4</v>
+      </c>
+      <c r="K28" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46146</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>46044</v>
+        <v>46188</v>
       </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -2078,7 +1810,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
@@ -2089,7 +1821,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2105,10 +1837,10 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>538.7</v>
+        <v>686</v>
       </c>
       <c r="K29" t="n">
-        <v>538.7</v>
+        <v>686</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -2118,17 +1850,17 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -2139,12 +1871,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>N</t>
@@ -2152,48 +1882,46 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K30" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -2204,12 +1932,12 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46033.86975694444</v>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" s="2" t="n">
-        <v>46037</v>
-      </c>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>N</t>
@@ -2217,7 +1945,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2241,12 +1969,12 @@
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>46034</v>
+        <v>46068</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2258,10 +1986,660 @@
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46064.87337962963</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0012-26</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>603</v>
+      </c>
+      <c r="K32" t="n">
+        <v>603</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46062.51478009259</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0011-26</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M33" t="n">
+        <v>-90.10947400000001</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46058.58436342593</v>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" s="2" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0009-26</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>585</v>
+      </c>
+      <c r="K34" t="n">
+        <v>869</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>46061</v>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>10'6" draft, 6 barges wide</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46051.75101851852</v>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" s="2" t="n">
+        <v>46061</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0008-26</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>303</v>
+      </c>
+      <c r="K35" t="n">
+        <v>869</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46050.44465277778</v>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" s="2" t="n">
+        <v>46052</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0007-26</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>303</v>
+      </c>
+      <c r="K36" t="n">
+        <v>585</v>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46045.53974537037</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>303</v>
+      </c>
+      <c r="K37" t="n">
+        <v>585</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0004-26</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>dredging</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M38" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46037.53365740741</v>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>shoaling</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="K39" t="n">
+        <v>538.7</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>303</v>
+      </c>
+      <c r="K40" t="n">
+        <v>869</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>303</v>
+      </c>
+      <c r="K41" t="n">
+        <v>869</v>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-01: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:U42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,19 +541,19 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -569,20 +569,20 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
@@ -608,25 +608,29 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -649,21 +653,21 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -686,21 +690,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -723,21 +727,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -760,21 +764,21 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -797,21 +801,21 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -834,21 +838,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -871,21 +875,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -904,29 +908,25 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -945,25 +945,29 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -986,21 +990,21 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1023,21 +1027,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1047,46 +1051,34 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K15" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1096,9 +1088,17 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K16" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1107,116 +1107,104 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>736</v>
-      </c>
-      <c r="K17" t="n">
-        <v>736</v>
-      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K18" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
+      <c r="N18" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
@@ -1227,113 +1215,125 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K19" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>785</v>
+      </c>
+      <c r="K20" t="n">
+        <v>785</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
+      <c r="N20" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -1344,67 +1344,55 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K21" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1414,9 +1402,17 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K22" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -1425,13 +1421,13 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -1442,136 +1438,128 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>849</v>
-      </c>
-      <c r="K23" t="n">
-        <v>849</v>
-      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K24" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
+      <c r="N24" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1583,14 +1571,14 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K25" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
@@ -1600,13 +1588,13 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -1617,124 +1605,120 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M26" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N26" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K26" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B27" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K27" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M27" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -1745,61 +1729,53 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K28" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O28" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1810,57 +1786,61 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K29" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1871,37 +1851,37 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K30" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
@@ -1911,17 +1891,17 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1932,11 +1912,9 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
@@ -1945,48 +1923,46 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K31" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1997,23 +1973,25 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B32" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -2024,30 +2002,32 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K32" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2058,65 +2038,57 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N33" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O33" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J33" t="n">
+        <v>603</v>
+      </c>
+      <c r="K33" t="n">
+        <v>603</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2127,12 +2099,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B34" t="inlineStr"/>
-      <c r="C34" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>N</t>
@@ -2140,48 +2110,54 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>585</v>
-      </c>
-      <c r="K34" t="n">
-        <v>869</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M34" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N34" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2192,11 +2168,11 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B35" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2205,7 +2181,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2221,7 +2197,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K35" t="n">
         <v>869</v>
@@ -2229,7 +2205,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
@@ -2239,14 +2215,14 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2257,11 +2233,11 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2270,7 +2246,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2289,17 +2265,17 @@
         <v>303</v>
       </c>
       <c r="K36" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -2311,7 +2287,7 @@
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2322,11 +2298,11 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2335,7 +2311,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2359,7 +2335,7 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
@@ -2376,7 +2352,7 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2387,10 +2363,12 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>N</t>
@@ -2398,54 +2376,48 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M38" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J38" t="n">
+        <v>303</v>
+      </c>
+      <c r="K38" t="n">
+        <v>585</v>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2456,57 +2428,65 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K39" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2517,25 +2497,23 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2546,32 +2524,30 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K40" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N40" t="inlineStr"/>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2582,11 +2558,11 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2595,7 +2571,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2619,12 +2595,12 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -2636,10 +2612,75 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>303</v>
+      </c>
+      <c r="K42" t="n">
+        <v>869</v>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-02: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,19 +541,19 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -569,32 +569,32 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>TX, LA - GULF OF AMERICA</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -610,20 +610,20 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>TX, LA - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
@@ -649,25 +649,29 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -690,21 +694,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -727,21 +731,21 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -764,21 +768,21 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -801,21 +805,21 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -838,21 +842,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -875,21 +879,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -912,21 +916,21 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -945,29 +949,25 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -986,25 +986,29 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1027,21 +1031,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1064,21 +1068,21 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1088,46 +1092,34 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K16" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1137,9 +1129,17 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>661.7</v>
+      </c>
+      <c r="K17" t="n">
+        <v>661.7</v>
+      </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1148,116 +1148,104 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>736</v>
-      </c>
-      <c r="K18" t="n">
-        <v>736</v>
-      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="K19" t="n">
-        <v>435.8</v>
+        <v>736</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
+      <c r="N19" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>46257</v>
+      </c>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
@@ -1268,113 +1256,125 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="K20" t="n">
-        <v>785</v>
+        <v>435.8</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" s="2" t="n">
-        <v>46244</v>
-      </c>
-      <c r="O20" s="2" t="n">
-        <v>46251</v>
-      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>785</v>
+      </c>
+      <c r="K21" t="n">
+        <v>785</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="N21" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Osceola Harbor</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1385,67 +1385,55 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>325.2</v>
-      </c>
-      <c r="K22" t="n">
-        <v>325.2</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1455,9 +1443,17 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>325.2</v>
+      </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
@@ -1466,13 +1462,13 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>WHITE RIVER</t>
+          <t>ARKANSAS RIVER</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1483,136 +1479,128 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>849</v>
-      </c>
-      <c r="K24" t="n">
-        <v>849</v>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>WHITE RIVER</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="K25" t="n">
-        <v>867</v>
+        <v>849</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46216.73908564815</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1624,14 +1612,14 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>10.3</v>
+        <v>857</v>
       </c>
       <c r="K26" t="n">
-        <v>10.3</v>
+        <v>867</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
@@ -1641,13 +1629,13 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1658,124 +1646,120 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.4634375</v>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M27" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N27" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>46195</v>
-      </c>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46160.52664351852</v>
-      </c>
-      <c r="B28" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="K28" t="n">
-        <v>777.7</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M28" t="n">
+        <v>-90.17319999999999</v>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="O28" s="2" t="n">
+        <v>46195</v>
+      </c>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Mouth of McKellar Lake</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1786,61 +1770,53 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46146.4284375</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>125.4</v>
+        <v>777.7</v>
       </c>
       <c r="K29" t="n">
-        <v>155.9</v>
+        <v>777.7</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" s="2" t="n">
-        <v>46146</v>
-      </c>
-      <c r="O29" s="2" t="n">
-        <v>46188</v>
-      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
-        </is>
-      </c>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -1851,57 +1827,61 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J30" t="n">
-        <v>686</v>
+        <v>125.4</v>
       </c>
       <c r="K30" t="n">
-        <v>686</v>
+        <v>155.9</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
+      <c r="N30" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O30" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Along RDB</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1912,37 +1892,37 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46119.48518518519</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="K31" t="n">
-        <v>348.7</v>
+        <v>686</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1952,17 +1932,17 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Along RDB</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1973,11 +1953,9 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46093.45828703704</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
@@ -1986,48 +1964,46 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>303</v>
+        <v>348.7</v>
       </c>
       <c r="K32" t="n">
-        <v>869</v>
+        <v>348.7</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Mid channel</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>"Possible shoaling," transit area with caution</t>
+        </is>
+      </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2038,23 +2014,25 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46064.87337962963</v>
-      </c>
-      <c r="B33" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -2065,30 +2043,32 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>603</v>
+        <v>303</v>
       </c>
       <c r="K33" t="n">
-        <v>603</v>
+        <v>869</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" s="2" t="n">
+        <v>46068</v>
+      </c>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>400 ft of green buoy line, near RDB</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2099,65 +2079,57 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46062.51478009259</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M34" t="n">
-        <v>-90.10947400000001</v>
-      </c>
-      <c r="N34" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O34" s="2" t="n">
-        <v>46065</v>
-      </c>
+      <c r="J34" t="n">
+        <v>603</v>
+      </c>
+      <c r="K34" t="n">
+        <v>603</v>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Amrize Dock on Mckellar Lake</t>
+          <t>400 ft of green buoy line, near RDB</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2168,12 +2140,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B35" t="inlineStr"/>
-      <c r="C35" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>N</t>
@@ -2181,48 +2151,54 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>585</v>
-      </c>
-      <c r="K35" t="n">
-        <v>869</v>
-      </c>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N35" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2233,11 +2209,11 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" s="2" t="n">
-        <v>46061</v>
+        <v>46068</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2246,7 +2222,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2262,7 +2238,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K36" t="n">
         <v>869</v>
@@ -2270,7 +2246,7 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
@@ -2280,14 +2256,14 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2298,11 +2274,11 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" s="2" t="n">
-        <v>46052</v>
+        <v>46061</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2311,7 +2287,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2330,17 +2306,17 @@
         <v>303</v>
       </c>
       <c r="K37" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -2352,7 +2328,7 @@
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2363,11 +2339,11 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="2" t="n">
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2376,7 +2352,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2400,7 +2376,7 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="2" t="n">
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
@@ -2417,7 +2393,7 @@
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2428,10 +2404,12 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>N</t>
@@ -2439,54 +2417,48 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J39" t="n">
+        <v>303</v>
+      </c>
+      <c r="K39" t="n">
+        <v>585</v>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O39" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46045</v>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2497,57 +2469,65 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="K40" t="n">
-        <v>538.7</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-90.10785143484679</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>46044</v>
+      </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Along LDB</t>
+          <t>McKellar Lake, near west side of Treasure Island</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>Transit the area with caution</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2558,25 +2538,23 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2587,32 +2565,30 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K41" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2623,11 +2599,11 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.50987268519</v>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" s="2" t="n">
-        <v>46037</v>
+        <v>46045</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2636,7 +2612,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0003-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2660,12 +2636,12 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" s="2" t="n">
-        <v>46034</v>
+        <v>46037</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
-          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -2677,10 +2653,75 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>303</v>
+      </c>
+      <c r="K43" t="n">
+        <v>869</v>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
+        <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-03: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U43"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,14 +541,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -569,32 +569,32 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -616,21 +616,21 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -651,32 +651,32 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -690,25 +690,29 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -727,25 +731,29 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -768,21 +776,21 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -805,21 +813,21 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -842,21 +850,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -879,21 +887,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -916,21 +924,21 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -953,21 +961,21 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -986,29 +994,25 @@
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1031,21 +1035,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1064,25 +1068,29 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1105,21 +1113,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1129,46 +1137,34 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K17" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1187,65 +1183,49 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J19" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K19" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
@@ -1256,25 +1236,21 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1284,17 +1260,9 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K20" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
@@ -1303,24 +1271,20 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
@@ -1331,7 +1295,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1351,30 +1315,30 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K21" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -1385,113 +1349,137 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K22" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K23" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
+      <c r="N23" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1505,102 +1493,82 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K25" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1610,17 +1578,9 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>857</v>
-      </c>
-      <c r="K26" t="n">
-        <v>867</v>
-      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
@@ -1629,13 +1589,13 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -1646,161 +1606,155 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K27" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
+      <c r="N27" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M28" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N28" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O28" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J28" t="n">
+        <v>857</v>
+      </c>
+      <c r="K28" t="n">
+        <v>867</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K29" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
@@ -1808,28 +1762,30 @@
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B30" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
@@ -1838,50 +1794,54 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K30" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M30" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -1892,7 +1852,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
@@ -1903,7 +1863,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1919,10 +1879,10 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K31" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1930,19 +1890,15 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -1953,7 +1909,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
@@ -1964,12 +1920,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1980,30 +1936,34 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K32" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
+      <c r="N32" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O32" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -2014,25 +1974,23 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -2043,32 +2001,30 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K33" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2079,37 +2035,37 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K34" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -2119,17 +2075,17 @@
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2140,9 +2096,11 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B35" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
@@ -2151,54 +2109,48 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M35" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J35" t="n">
+        <v>303</v>
+      </c>
+      <c r="K35" t="n">
+        <v>869</v>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O35" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2209,25 +2161,23 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B36" t="inlineStr"/>
-      <c r="C36" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -2238,32 +2188,30 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K36" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N36" t="inlineStr"/>
       <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2274,12 +2222,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B37" t="inlineStr"/>
-      <c r="C37" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>N</t>
@@ -2287,48 +2233,54 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>303</v>
-      </c>
-      <c r="K37" t="n">
-        <v>869</v>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M37" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N37" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2339,11 +2291,11 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2352,7 +2304,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2368,32 +2320,32 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K38" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2404,11 +2356,11 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B39" t="inlineStr"/>
       <c r="C39" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2417,7 +2369,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2436,17 +2388,17 @@
         <v>303</v>
       </c>
       <c r="K39" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -2458,7 +2410,7 @@
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2469,10 +2421,12 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>N</t>
@@ -2480,54 +2434,48 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J40" t="n">
+        <v>303</v>
+      </c>
+      <c r="K40" t="n">
+        <v>585</v>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O40" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2538,23 +2486,25 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -2565,30 +2515,32 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K41" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
+      <c r="N41" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2599,12 +2551,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B42" t="inlineStr"/>
-      <c r="C42" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>N</t>
@@ -2612,48 +2562,54 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>303</v>
-      </c>
-      <c r="K42" t="n">
-        <v>869</v>
-      </c>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M42" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N42" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2664,25 +2620,23 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2693,35 +2647,163 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K43" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" s="2" t="n">
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>303</v>
+      </c>
+      <c r="K44" t="n">
+        <v>869</v>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>303</v>
+      </c>
+      <c r="K45" t="n">
+        <v>869</v>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr">
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
+      <c r="Q45" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr">
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Daily pipeline 2026-09-04: new data pending review
</commit_message>
<xml_diff>
--- a/notices_2026.xlsx
+++ b/notices_2026.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U45"/>
+  <dimension ref="A1:U47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,26 +541,34 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46268.45350694445</v>
+        <v>46268.97141203703</v>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0096-26</t>
+          <t>SEC LMR BNM 0055-26</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>303</v>
+      </c>
+      <c r="K2" t="n">
+        <v>869</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
@@ -569,27 +577,27 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>TX - GULF OF AMERICA</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
+          <t>Mariners be advised of MSIB 26-10 which updates low-water restrictions on September 7th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:• Barge drafts not to exceed 11’6”.• Barge configurations not to exceed 7 wide.For Southbound traffic MM 585-303:• Barge drafts not to exceed 12’6”.• Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:• Barge drafts shall not exceed 10’6”.• Barge configurations not to exceed 4 wide and 6 long max on loads.• Barge configurations not to exceed 6 wide and 7 long overall. BT</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46267.53146990741</v>
+        <v>46268.53527777778</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0095-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -608,29 +616,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>TX, LA - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0054-26 DTG 211819Z AUG 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46267.39673611111</v>
+        <v>46268.45350694445</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0094-26</t>
+          <t>CGD-H BNM 0096-26</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -651,32 +655,32 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>AL - GULF OF AMERICA</t>
+          <t>TX - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
+          <t>FROM 03SEP2026 TO 17SEP2026, THE M/V GALVESTON AND TRITONCRUSADER WILL CONDUCT DIVING OPERATIONS IN THE GALVESTON ENTRANCE SAFETY FAIRWAY IN APPROXIMATE POSITION 29-10-52.1N 094-31-13.1W, WITH ANCHORS SET IN APPROXIMATE POSITIONS 29-11-11.5N 094-31-22.9W AND 29-10-37.4N 094-31-15.9W. MARINERS ARE URGED TO TRANSIT THE AREA WITH CAUTION. CANCEL AT//180500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46266.39112268519</v>
+        <v>46267.53146990741</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0093-26</t>
+          <t>CGD-H BNM 0095-26</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -698,21 +702,21 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
+          <t>DUE TO THE PASSAGE OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION, STRUCTURES OR PLATFORMS IN THE GULF OF AMERICA AND SURROUNDING WATERS, MAY BE DAMAGED, DESTROYED OR SUBMERGED. BUOYS MAY HAVE MOVED FROM ASSIGNED POSITIONS, BE DAMAGED, EXTINGUISHED, SUNK, OR OTHERWISE MADE INOPERATIVE. MARINERS SHOULD NOT SOLELY RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN THESE AREAS, BUT SHOULD EMPLOY SUCH OTHER AVAILABLE METHODS OF DETERMINING POSITION. WRECKS, SUBMERGED OBSTRUCTIONS AND PIPELINES MAY MOVE FROM CHARTED LOCATIONS OR BECOME UNCOVERED DUE TO THE FORCE OF STORM SURGE. MARINERS ARE URGED TO USE EXTREME CAUTION AND REPORT ALL AIDS TO NAVIGATION DISCREPANCIES AND HAZARDS TO THE NEAREST U.S. COAST GUARD UNIT. BT</t>
         </is>
       </c>
       <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46265.53005787037</v>
+        <v>46267.39673611111</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0094-26</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -733,32 +737,32 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
+          <t>ON 03SEP2026, FROM 2130Z TO 0030Z, ON 04SEP2026, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//040130Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46265.52835648148</v>
+        <v>46266.39112268519</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SEC LMR</t>
+          <t>CGD-H BNM 0093-26</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -772,25 +776,29 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>TX, LA - GULF OF AMERICA</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
+          <t>1. WITH THE APPROACH OF TROPICAL STORM EDOUARD, AIDS TO NAVIGATION AND STRUCTURES IN THE GULF OF AMERICA AND SURROUNDING WATERS MAY BE DAMAGED OR DESTROYED. LIGHTED AND UNLIGHTED BUOYS MAY MOVE FROM ASSIGNED POSITIONS, SINK, BE DAMAGED, EXTINGUISHED, OR MADE INOPERATIVE. MARINERS SHOULD NOT RELY UPON THE POSITION OR OPERATION OF AN AID TO NAVIGATION IN AFFECTED AREAS, AND SHOULD EMPLOY OTHER METHODS FOR DETERMINING POSITION. WRECKS AND SUBMERGED OBSTRUCTIONS MAY MOVE FROM CHARTED LOCATIONS AND PIPELINES MAY BECOME UNCOVERED OR MOVE DUE TO STORM SURGES. STORM SURGE AND WINDS MAY CREATE SHOALS IN AFFECTED WATERS. DRAWBRIDGES MAY DEVIATE FROM NORMAL OPERATING PROCEDURES AND MAY BE UNABLE TO OPEN DUE TO HIGH WINDS OR TO FACILITATE EVACUATION OF LAND TRAFFIC. MARINERS SHOULD ANTICIPATE BRIDGE CLOSURES BY LISTENING TO THE NATIONAL WEATHER SERVICE AND COAST GUARD BROADCASTS ON TROPICAL STORM CONDITIONS. LOCKS AND NAVIGATION STRUCTURES WILL PASS NAVIGATION UNTIL WATER LEVELS AND WIND CONDITIONS WARRANT OPERATIONS UNSAFE. THE STRUCTURES WILL THEN CLOSE IN ACCORDANCE WITH HURRICANE PROCEDURES. MARINERS WILL BE GIVEN AS MUCH NOTICE AS POSSIBLE WHEN STRUCTURES ARE TOO CLOSE; HOWEVER, STRUCTURES MAY CLOSE ON SHORT NOTICE OR WELL IN ADVANCE OF THE ACTUAL STORM. DUE TO THE UNCERTAINTY REGARDING TROPICAL STORM MOVEMENTS AND BRIDGE AND STRUCTURE CLOSURES, MARINERS SHOULD SEEK PASSAGE AND SAFE HARBOR AS SOON AS POSSIBLE AND WELL IN ADVANCE OF THE ARRIVAL OF GALE FORCE WINDS.CANCEL AT//021330Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46265.52792824074</v>
+        <v>46265.53005787037</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0014-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -809,25 +817,29 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>SEC LMR</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. THE FOLLOWING SECTOR LOWER MISSISSIPPI BROADCAST NOTICE TO MARINERS ARE STILL IN EFFECT AS OF 311627Z AUG 26:A. SEC LMR BNM 0054-26 : SAFETY, ISSUED 211819Z AUG 26. 2. ALL OTHER SECTOR LOWER MISSISSIPPI BROADCAST NOTICES TO MARINERS ARE NO LONGER IN EFFECT OR HAVE BEEN INCLUDED IN THE LNM AS OF THE DATE-TIME IN PARAGRAPH 1. BTCANCEL MESSAGES: {SEC LMR BNM 0034-24 DTG 041926Z OCT 24, SEC LMR BNM 0057-25 DTG 111905Z AUG 25, SEC LMR BNM 0074-25 DTG 151522Z SEP 25, SEC LMR BNM 0088-25 DTG 142010Z OCT 25, SEC LMR BNM 0071-25 DTG 011419Z SEP 25}</t>
         </is>
       </c>
       <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265.52695601852</v>
+        <v>46265.52835648148</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -850,21 +862,21 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>CANCEL MESSAGES: {SEC LMR BNM 0014-26 DTG 120047Z FEB 26, SEC LMR BNM 0053-25 DTG 011528Z AUG 25, SEC LMR BNM 0013-25 DTG 241726Z FEB 25, SEC LMR BNM 0042-24 DTG 041724Z NOV 24, SEC LMR BNM 0025-25 DTG 291633Z APR 25, SEC LMR BNM 0115-25 DTG 172120Z DEC 25}</t>
         </is>
       </c>
       <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46265.52664351852</v>
+        <v>46265.52792824074</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0014-26</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -887,21 +899,21 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0014-26 DTG 120047Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46265.52623842593</v>
+        <v>46265.52695601852</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -924,21 +936,21 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0044-26 DTG 131415Z JUL 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46265.52559027778</v>
+        <v>46265.52664351852</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -961,21 +973,21 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46265.52508101852</v>
+        <v>46265.52623842593</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -998,21 +1010,21 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
+          <t>1. CANCEL SEC LMR BNM 0021-26 DTG 071509Z APR 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46265.52371527778</v>
+        <v>46265.52559027778</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0107-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1035,21 +1047,21 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
+          <t>1. CANCEL SEC LMR BNM 0107-26 DTG 130806Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46265.42929398148</v>
+        <v>46265.52508101852</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0092-26</t>
+          <t>SEC LMR BNM 0106-26 (CORRECTION)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1068,29 +1080,25 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
-        </is>
-      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0106-26 DTG 112246Z JAN 26 BT</t>
         </is>
       </c>
       <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46258.44554398148</v>
+        <v>46265.52371527778</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0087-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1113,21 +1121,21 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0012-26 DTG 120042Z FEB 26A. AID NAME:B. LLNR:C. SUPERCEDED BY:D. COMMENTS: BT</t>
         </is>
       </c>
       <c r="U16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46258.44363425926</v>
+        <v>46265.42929398148</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0086-26</t>
+          <t>CGD-H BNM 0092-26</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1146,25 +1154,29 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>LA - GULF OF AMERICA - SOUTHWEST PASS</t>
+        </is>
+      </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
+          <t>UNMANNED SURFACE VESSEL (USV) OPERATIONS ARE TAKING PLACE ADJACENT TO AND WEST OF THE SW PASS ENTRANCE CHANNEL BY THE USV MC29, IN AN AREA BOUND BY APPROXIMATE POSITIONS:28-54-12N 089-27-15W,28-54-12N 089-26-00W,28-51-01N 089-26-00W AND28-51-01N 089-27-15W. MARINERS ARE URGED TO MAINTAIN A WIDE BERTH FROM THE USV. CANCEL AT//060500Z SEP 26// BT</t>
         </is>
       </c>
       <c r="U17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46257.8184375</v>
+        <v>46258.44554398148</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>CGD-H BNM 0087-26</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1187,21 +1199,21 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
+          <t>1. CANCEL CGD-H BNM 0087-26 DTG 141803Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46255.75466435185</v>
+        <v>46258.44363425926</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0054-26</t>
+          <t>CGD-H BNM 0086-26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1211,46 +1223,34 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>661.7</v>
-      </c>
-      <c r="K19" t="n">
-        <v>661.7</v>
-      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
-        </is>
-      </c>
+      <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. CANCEL CGD-H BNM 0086-26 DTG 141758Z AUG 262. OPERATION COMPLETE. BT</t>
         </is>
       </c>
       <c r="U19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46253.46241898148</v>
+        <v>46257.8184375</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CGD-H BNM 0091-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1269,65 +1269,49 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>AL - GULF OF AMERICA</t>
-        </is>
-      </c>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
-          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+          <t>1. CANCEL SEC LMR BNM 0053-26 DTG 171544Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46251.58453703704</v>
+        <v>46255.75466435185</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0053-26</t>
+          <t>SEC LMR BNM 0054-26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="K21" t="n">
-        <v>736</v>
+        <v>661.7</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" s="2" t="n">
-        <v>46251</v>
-      </c>
-      <c r="O21" s="2" t="n">
-        <v>46257</v>
-      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
@@ -1338,25 +1322,21 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+          <t>1.  MARINERS BE ADVISED THAT THE NAVIGATION LIGHTS ON THE HELENA BRIDGE MM 661.7 LMR ARE NOT WORKING. 2.  MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46245.37090277778</v>
+        <v>46253.46241898148</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0052-26</t>
+          <t>CGD-H BNM 0091-26</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1366,17 +1346,9 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J22" t="n">
-        <v>435.8</v>
-      </c>
-      <c r="K22" t="n">
-        <v>435.8</v>
-      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
@@ -1385,24 +1357,20 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>AL - GULF OF AMERICA</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>ON 21AUG2026, FROM 1600Z TO 2300Z, A LIVE FIRE EXERCISE WILL BE HELD IN THE GULF OF AMERICA, W-155A4, BOUND BY APPROXIMATE POSITIONS:30-10-01N 088-01-30W, 30-11-21N 087-44-15W,30-09-45N 087-45-47W,30-04-03N 087-41-17W,30-02-53N 087-42-16W,30-00-01N 087-38-32W,30-00-00N 088-01-30W AND30-10-00N 088-01-30W.THE AREA OF HAZARD IS SURFACE TO 5,000 FEET. MARINERS ARE URGED TO REMAIN CLEAR OF THE AREA DURING THE EXERCISEPERIOD.CANCEL AT//212359Z AUG 26// BT</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46244.33856481482</v>
+        <v>46251.58453703704</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
@@ -1413,7 +1381,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0051-26</t>
+          <t>SEC LMR BNM 0053-26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1433,30 +1401,30 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="K23" t="n">
-        <v>785</v>
+        <v>736</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="O23" s="2" t="n">
-        <v>46251</v>
+        <v>46257</v>
       </c>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Osceola Harbor</t>
+          <t>LOWER MISSISSIPPI RIVER</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT LMR MM 736 ON THE LDB FROM AUGUST 17TH THROUGH 23RD.2. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK AND PROCEED AT SLOW BELL.3. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 13, CHANNEL 71, OR VIA TELEPHONE AT314-550-0520.4. CANCEL AT TIME//230800L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -1467,113 +1435,137 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46244.30862268519</v>
+        <v>46245.37090277778</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0052-26</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">cancellation </t>
+          <t>other</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>435.8</v>
+      </c>
+      <c r="K24" t="n">
+        <v>435.8</v>
+      </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
-          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
+          <t>LOWER MISSISSIPPI RIVER MM 435.8   1.THE SECOND ALTERNATE SPAN OF THE VICKSBURG (I-20) BRIDGE, CLOSEST TO THE RDB, IS CLOSED DUE TO LOW WATER.   2.MARINERS SHOULD TRANSIT THE VICKSBURG BRIDGE USING THE MAIN SPAN OR FIRST ALTERNATE SPAN.  BT</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46239.68305555556</v>
+        <v>46244.33856481482</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0050-26</t>
+          <t>SEC LMR BNM 0051-26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="K25" t="n">
-        <v>325.2</v>
+        <v>785</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
+      <c r="N25" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>46251</v>
+      </c>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
+          <t>Osceola Harbor</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
+          <t>1. DREDGING WILL TAKE PLACE AT OSCEOLA HARBOR FROM AUGUST 10TH THROUGH 17TH, IVO LMR MM 785. EXERCISE CAUTION WHEN IN VICINITY OF THE WORK.2. FOR MORE INFORMATION, CONTACT DREDGE MIDWAY ON CHANNEL 10 OR CHANNEL 71. BT</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46238.74310185185</v>
+        <v>46244.30862268519</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0049-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t xml:space="preserve">cancellation </t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1587,102 +1579,82 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>WHITE RIVER</t>
-        </is>
-      </c>
+      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
+          <t>1. CANCEL SEC LMR BNM 0046-26 DTG 010055Z AUG 26 BT</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46234.89293981482</v>
+        <v>46239.68305555556</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0046-26</t>
+          <t>SEC LMR BNM 0050-26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J27" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="K27" t="n">
-        <v>849</v>
+        <v>325.2</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" s="2" t="n">
-        <v>46234</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>46243</v>
-      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>TRANSIT THE AREA WITH CAUTION</t>
-        </is>
-      </c>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr">
         <is>
-          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>1. RED BUOY WAS REPORTED PARTIALLY SUBMERGED IVO ARKANSAS RIVER MM 325.2. MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION.BT BT</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46216.73908564815</v>
+        <v>46238.74310185185</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0045-26</t>
+          <t>SEC LMR BNM 0049-26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1692,17 +1664,9 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LMR</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>857</v>
-      </c>
-      <c r="K28" t="n">
-        <v>867</v>
-      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
@@ -1711,13 +1675,13 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
-          <t>LOWER MISSISSIPPI RIVER</t>
+          <t>WHITE RIVER</t>
         </is>
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
+          <t>1. MARINERS BE ADVISED OF HIGH DIFFERENTIAL AT WHITE RIVER ENTRANCE CHANNEL STARTING AUGUST 6TH. EXERCISE EXTREME CAUTION WHEN PASSING THROUGH MONTGOMERY POINT LOCK AND DAM. CONTACT THE LOCK OPERATOR FOR LATEST INFORMATION VIA VHF OR 870-548-3400.2. CANCEL AT TIME// 100900L AUG 26//. BT</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -1728,161 +1692,155 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46216.4634375</v>
+        <v>46234.89293981482</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0044-26</t>
+          <t>SEC LMR BNM 0046-26</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>LMR</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="K29" t="n">
-        <v>10.3</v>
+        <v>849</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+      <c r="N29" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>46243</v>
+      </c>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr">
         <is>
-          <t>ARKANSAS RIVER</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>TRANSIT THE AREA WITH CAUTION</t>
+        </is>
+      </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1. DREDGE MIDWAY WILL BE CONDUCTING DREDGING OPERATIONS INTERMITTENLY INVO MM 849 LMR UNTIL AUGUST 9TH. THE DREDGE MIDWAY CAN BE REACHED ON CHANNEL 13 OR 71 2. ALL MARINERS ARE ADVISED TO TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46186.8905787037</v>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>46199</v>
-      </c>
+        <v>46216.73908564815</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0039-26</t>
+          <t>SEC LMR BNM 0045-26</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="n">
-        <v>35.07917</v>
-      </c>
-      <c r="M30" t="n">
-        <v>-90.17319999999999</v>
-      </c>
-      <c r="N30" s="2" t="n">
-        <v>46188</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>46195</v>
-      </c>
+      <c r="J30" t="n">
+        <v>857</v>
+      </c>
+      <c r="K30" t="n">
+        <v>867</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Mouth of McKellar Lake</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+          <t>LOWER MISSISSIPPI RIVER</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
+          <t>1. MARINERS ARE ADVISED THAT M/V HOU. RIVERS WILL BE WORKING AT MM 857 LOWER MISSISSIPPI RIVER LDB 13JUL-13AUG2. BEGINING 19JUL THROUGH 30JUL THE AREA WILL BE CLOSED TO SOUTHBOUND TRAFFIC FOR TOWS OF 20 OR MORE BARGES3. VESSELS TRANSITING THE AREA ARE REQUESTED TO CONTACT VESSEL HOU. RIVERS TO CHECK IN AT SOUTHBOUND AT MM 8674. VESSEL HOU. RIVERS MAY BE CONTACTED FOR CHECK IN VIA MARINE VHF-FM CH-13, CH-16 and CH-72 OR VIA TELEPHONE AT 573-841-0984 BT</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46160.52664351852</v>
+        <v>46216.4634375</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0032-26</t>
+          <t>SEC LMR BNM 0044-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="K31" t="n">
-        <v>777.7</v>
+        <v>10.3</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
@@ -1890,28 +1848,30 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>Proceed with caution</t>
-        </is>
-      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>ARKANSAS RIVER</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr">
         <is>
-          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
+          <t>1. Mariners should expect to experience intermittent delays at Norrell Lock (No. 1) MM 10.3 ARK July 13, 2026 - July 17, 2026, between the hours of 6:00 a.m. and 6:00 p.m. The intermittent delays are required to facilitate work on the hydraulic system.2. Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46146.4284375</v>
-      </c>
-      <c r="B32" t="inlineStr"/>
+        <v>46186.8905787037</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>46199</v>
+      </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
@@ -1920,50 +1880,54 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0029-26</t>
+          <t>SEC LMR BNM 0039-26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>other_dredging</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>ARK</t>
-        </is>
-      </c>
-      <c r="J32" t="n">
-        <v>125.4</v>
-      </c>
-      <c r="K32" t="n">
-        <v>155.9</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="n">
+        <v>35.07917</v>
+      </c>
+      <c r="M32" t="n">
+        <v>-90.17319999999999</v>
+      </c>
       <c r="N32" s="2" t="n">
-        <v>46146</v>
+        <v>46188</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
+          <t>Mouth of McKellar Lake</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING AT THE MOUTH OF MCKELLAR LAKE, FROM JUNE 15TH THROUGH 22ND. THE CHANNEL WILL BE BLOCKED DURING OPERATIONS. 2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM. 3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71. 4.CANCEL AT TIME//221200 FEB 26//. BT</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -1974,7 +1938,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46119.48518518519</v>
+        <v>46160.52664351852</v>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
@@ -1985,7 +1949,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0021-26</t>
+          <t>SEC LMR BNM 0032-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2001,10 +1965,10 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="K33" t="n">
-        <v>686</v>
+        <v>777.7</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
@@ -2012,19 +1976,15 @@
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Along RDB</t>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr">
         <is>
-          <t>Maintain safe distance from buoy line and transit with caution</t>
+          <t>Proceed with caution</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
+          <t>LMR MM 777.71. COAST GUARD RECEIVED A REPORT OF SHOALING AT MM 777.7 LMR2. MARINERS ARE ADVISED TO PROCEED WITH CAUTION BT</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -2035,7 +1995,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46093.45828703704</v>
+        <v>46146.4284375</v>
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr"/>
@@ -2046,12 +2006,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0018-26</t>
+          <t>SEC LMR BNM 0029-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>other_shoaling</t>
+          <t>other_dredging</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -2062,30 +2022,34 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>348.7</v>
+        <v>125.4</v>
       </c>
       <c r="K34" t="n">
-        <v>348.7</v>
+        <v>155.9</v>
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+      <c r="N34" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="O34" s="2" t="n">
+        <v>46188</v>
+      </c>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Mid channel</t>
+          <t>Murray Lock (No. 7) to Toad Suck Lock (No. 8)</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>"Possible shoaling," transit area with caution</t>
+          <t>Intermittent delays for dredging and dive inspections in preparation of the 110' stoplog conversions</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
+          <t>1.Mariners may experience intermittent delays at Murray Lock (No. 7) MM 125.4 ARK and Toad Suck Lock (No. 8) MM 155.9 on May 4th, 2026 through June 15th, 2026 between the hours of 7:00 a.m. and 5:30 p.m. daily.2.The intermittent delays are required to facilitate dredging and dive inspections in preparation of the 110' stoplog conversions.3.Questions or requests for additional information concerning this notice should be directed to the Little Rock District Office, at (501) 324-5096 or you may email CESWL-OP-OM@usace.army.mil. BT</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -2096,25 +2060,23 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46065.67140046296</v>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>46070</v>
-      </c>
+        <v>46119.48518518519</v>
+      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0015-26</t>
+          <t>SEC LMR BNM 0021-26</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -2125,32 +2087,30 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>303</v>
+        <v>686</v>
       </c>
       <c r="K35" t="n">
-        <v>869</v>
+        <v>686</v>
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Along RDB</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Maintain safe distance from buoy line and transit with caution</t>
+        </is>
+      </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. SHOALING HAS BEEN REPORTED ALONG THE RDB AT MM 686 LMR.2. MARINERS ARE ADVISED TO MAINTAIN A SAFE DISTANCE FROM THE BUOY LINE AND TRANSIT THE AREA WITH CAUTION. BT</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -2161,37 +2121,37 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46064.87337962963</v>
+        <v>46093.45828703704</v>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0012-26</t>
+          <t>SEC LMR BNM 0018-26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>other_shoaling</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>LMR</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="K36" t="n">
-        <v>603</v>
+        <v>348.7</v>
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -2201,17 +2161,17 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
-          <t>400 ft of green buoy line, near RDB</t>
+          <t>Mid channel</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Proceed with caution</t>
+          <t>"Possible shoaling," transit area with caution</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
+          <t>UNCLASSUBJ: SAFETY BROADCAST NOTICE TO MARINERSSEC LMR BNM 0018ARK 348.71.WRCC received notification of possible shoaling at MM 348.7 ARK mid channel.2. All mariners are advised to transit the area with caution. BT</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -2222,9 +2182,11 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46062.51478009259</v>
-      </c>
-      <c r="B37" t="inlineStr"/>
+        <v>46065.67140046296</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>46070</v>
+      </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
@@ -2233,54 +2195,48 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0011-26</t>
+          <t>SEC LMR BNM 0015-26</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="n">
-        <v>35.085769</v>
-      </c>
-      <c r="M37" t="n">
-        <v>-90.10947400000001</v>
-      </c>
+      <c r="J37" t="n">
+        <v>303</v>
+      </c>
+      <c r="K37" t="n">
+        <v>869</v>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>46065</v>
-      </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Amrize Dock on Mckellar Lake</t>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
-        </is>
-      </c>
+        <v>46068</v>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
+          <t>Mariners be advised that MSIB 26-08 updates low-water restrictions on February 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -2291,25 +2247,23 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46058.58436342593</v>
+        <v>46064.87337962963</v>
       </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" s="2" t="n">
-        <v>46068</v>
-      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0009-26</t>
+          <t>SEC LMR BNM 0012-26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
@@ -2320,32 +2274,30 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>585</v>
+        <v>603</v>
       </c>
       <c r="K38" t="n">
-        <v>869</v>
+        <v>603</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>10'6" draft, 6 barges wide</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>400 ft of green buoy line, near RDB</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Proceed with caution</t>
+        </is>
+      </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1. MARINERS BE ADVISED. SHOALING HAS BEEN REPORTED 400 FEET OF GREEN BUOY LINE AT MM 603 LMR, NEAR THE RDB.2. ALL MARINERS ARE ADVISED TO PROCEED WITH CAUTION WHILE TRANSITING THE AREA. FOR QUESTIONS OR CONCERNS PLEASE CONTACT WESTERN RIVERS COMMAND CENTER AT 1-866-360-3386. BT</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -2356,12 +2308,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46051.75101851852</v>
+        <v>46062.51478009259</v>
       </c>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" s="2" t="n">
-        <v>46061</v>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>N</t>
@@ -2369,48 +2319,54 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0008-26</t>
+          <t>SEC LMR BNM 0011-26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>303</v>
-      </c>
-      <c r="K39" t="n">
-        <v>869</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="n">
+        <v>35.085769</v>
+      </c>
+      <c r="M39" t="n">
+        <v>-90.10947400000001</v>
+      </c>
       <c r="N39" s="2" t="n">
-        <v>46052</v>
-      </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
+        <v>46062</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Amrize Dock on Mckellar Lake</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily </t>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>1.DREDGE MIDWAY WILL BE WORKING IVO AMRIZE DOCK ON MCKELLAR LAKE, NEAR THE WEST SIDE OF TREASURE ISLAND. WORK WILL BE FROM FEBRUARY 9TH THROUGH 12TH AND THE CHANNEL WILL BE BLOCKED DURING OPERATIONS.2.TRAFFIC WILL BE PERMITTED TO PASS DAILY FROM NOON TO 1PM AND MIDNIGHT TO 1AM.3.DREDGE MIDWAY CAN BE CONTACTED ON VHF CHANNEL 13 OR 71.4.CANCEL AT TIME// 130800 FEB 26//.CANCEL AT//130800Z FEB 26// BT</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -2421,11 +2377,11 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46050.44465277778</v>
+        <v>46058.58436342593</v>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" s="2" t="n">
-        <v>46052</v>
+        <v>46068</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2434,7 +2390,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0007-26</t>
+          <t>SEC LMR BNM 0009-26</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2450,32 +2406,32 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>303</v>
+        <v>585</v>
       </c>
       <c r="K40" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>11'6" draft, 7 barges wide</t>
+          <t>10'6" draft, 6 barges wide</t>
         </is>
       </c>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
+          <t>Mariners be advised that MSIB 26-07 updates low-water restrictions on February 8th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 10'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -2486,11 +2442,11 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46045.53974537037</v>
+        <v>46051.75101851852</v>
       </c>
       <c r="B41" t="inlineStr"/>
       <c r="C41" s="2" t="n">
-        <v>46050</v>
+        <v>46061</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2499,7 +2455,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0008-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2518,17 +2474,17 @@
         <v>303</v>
       </c>
       <c r="K41" t="n">
-        <v>585</v>
+        <v>869</v>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" s="2" t="n">
-        <v>46045</v>
+        <v>46052</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
-          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -2540,7 +2496,7 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr">
         <is>
-          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
+          <t>Mariners be advised of MSIB 26-06 which updates low-water restrictions on January 30th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'6".Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -2551,10 +2507,12 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46042.81428240741</v>
+        <v>46050.44465277778</v>
       </c>
       <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" s="2" t="n">
+        <v>46052</v>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>N</t>
@@ -2562,54 +2520,48 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0004-26</t>
+          <t>SEC LMR BNM 0007-26</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>dredging</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Midway</t>
-        </is>
-      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="n">
-        <v>35.0859560963022</v>
-      </c>
-      <c r="M42" t="n">
-        <v>-90.10785143484679</v>
-      </c>
+      <c r="J42" t="n">
+        <v>303</v>
+      </c>
+      <c r="K42" t="n">
+        <v>585</v>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" s="2" t="n">
-        <v>46042.81428240741</v>
-      </c>
-      <c r="O42" s="2" t="n">
-        <v>46044</v>
-      </c>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>McKellar Lake, near west side of Treasure Island</t>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
-        </is>
-      </c>
+        <v>46050</v>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
-          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-05 which updates low-water restrictions on January 28th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:Barge drafts not to exceed 11'6".Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:Barge drafts not to exceed 11'6".Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Barge drafts shall not exceed 10'.Barge configurations not to exceed 4 wide max on loads, 6 wide overall.Barge configurations not to exceed 7 long overall. BT</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -2620,23 +2572,25 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46037.53365740741</v>
+        <v>46045.53974537037</v>
       </c>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" s="2" t="n">
+        <v>46050</v>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
+          <t>SEC LMR BNM 0003-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>shoaling</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2647,30 +2601,32 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>538.7</v>
+        <v>303</v>
       </c>
       <c r="K43" t="n">
-        <v>538.7</v>
+        <v>585</v>
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
+      <c r="N43" s="2" t="n">
+        <v>46045</v>
+      </c>
       <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Along LDB</t>
-        </is>
-      </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>Transit the area with caution</t>
-        </is>
-      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>10' draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr">
         <is>
-          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+          <t>LMR 303-869Mariners be advised of MSIB 26-04 which updates low-water restrictions on January 23rd, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-585:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'6".â€¢ Barge configurations not to exceed 6 wide.For Southbound traffic MM 585-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 11'6".â€¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:â€¢ Effective January 23, 2026, barge drafts shall not exceed 10'.â€¢ Barge configurations not to exceed 4 wide max on loads, 6 wide overall.â€¢ Barge configurations not to exceed 7 long overall.* All barges in transit will be clear to proceed prior to January 23, 2026.* BT</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -2681,12 +2637,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46037.50987268519</v>
+        <v>46042.81428240741</v>
       </c>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" s="2" t="n">
-        <v>46045</v>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>N</t>
@@ -2694,48 +2648,54 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0003-26</t>
+          <t>SEC LMR BNM 0004-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>dredging</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Midway</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>LMR</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>303</v>
-      </c>
-      <c r="K44" t="n">
-        <v>869</v>
-      </c>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="n">
+        <v>35.0859560963022</v>
+      </c>
+      <c r="M44" t="n">
+        <v>-90.10785143484679</v>
+      </c>
       <c r="N44" s="2" t="n">
-        <v>46037</v>
-      </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>11'6" draft, 7 barges wide</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
+        <v>46042.81428240741</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>McKellar Lake, near west side of Treasure Island</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Traffic allowed: Noon-1pm, Midnight-1am daily, Traffic blocked on west side of Treasure Island</t>
+        </is>
+      </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+          <t>McKellar LakeDredge MIDWAY will be working IVO McKellar Lake near the west side of Treasure Island.The dredge pipeline will block traffic on the west side of Treasure Island until Thursday, 22JAN26.Dredge MIDWAY will pass traffic twice a day, noon to 1 pm and midnight to 1am.For any questions or concerns regarding the aforementioned dredge operations, please contact dredge MIDWAY on channel 13 or channel 71.BT</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -2746,25 +2706,23 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46033.86975694444</v>
+        <v>46037.53365740741</v>
       </c>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" s="2" t="n">
-        <v>46037</v>
-      </c>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>SEC LMR BNM 0106-26</t>
+          <t>SEC LMR BNM 0002-26 UPDATE-1</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>shoaling</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2775,35 +2733,163 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>303</v>
+        <v>538.7</v>
       </c>
       <c r="K45" t="n">
-        <v>869</v>
+        <v>538.7</v>
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" s="2" t="n">
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Along LDB</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Transit the area with caution</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>1. WRCC received notification of possible shoaling at MM 538.7 LMR along the LDB.2. All mariners are advised to transit the area with caution BT</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46037.50987268519</v>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0003-26</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>303</v>
+      </c>
+      <c r="K46" t="n">
+        <v>869</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>10'6" draft, 5 barges wide max on loads, 7 wide overall. Barge configurations not to exceed 7 long overall</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>11'6" draft, 7 barges wide</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Mariners be advised of MSIB 26-03 which updates low-water restrictions on January 15th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts not to exceed 11'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations not to exceed 5 wide max on loads, 7 wide overall.Ã¢â‚¬Â¢ Barge configurations not to exceed 7 long overall BT</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46033.86975694444</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" s="2" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SEC LMR BNM 0106-26</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>LMR</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>303</v>
+      </c>
+      <c r="K47" t="n">
+        <v>869</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" s="2" t="n">
         <v>46034</v>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr">
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr">
         <is>
           <t>10'6" draft, 4 barges wide max on loads, 6 wide overall. Barge configurations not to exceed 7 long overall</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="Q47" t="inlineStr">
         <is>
           <t>11'6" draft, 7 barges wide</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr">
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
         <is>
           <t>LMR MM 303-869Mariners be advised of MSIB 26-02 which updates low-water restrictions on January 12th, 2026, for MM 303-869 on the LMR. They are as follows:For Southbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 11'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 wide.For Northbound traffic MM 869-303:Ã¢â‚¬Â¢ Barge drafts shall not exceed 10'6".Ã¢â‚¬Â¢ Barge configurations shall not exceed 4 wide max on loads, 6 wide overall.Ã¢â‚¬Â¢ Barge configurations shall not exceed 7 long overall.BT</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="U47" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>